<commit_message>
fix: preserve native CPU guard and complete V163 validation controls
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -121,8 +121,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E31" totalsRowShown="0">
-  <autoFilter ref="A5:E31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E32" totalsRowShown="0">
+  <autoFilter ref="A5:E32"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2247,12 +2247,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2274,12 +2274,12 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Garantir l’activation native du bouton Retour au clavier et au pointeur sans modale de focus intermédiaire, libérer les commandes tenues et conserver la pause des champs ordinaires et du blur. Vérifier aussi les sorties spatiales et la reprise du dernier projectile Broodstorm par les vrais menus et sauvegardes.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requéraient une recette liée au candidat courant avec vrai parcours production/menu/Save. La preview production a ensuite reproduit un clic Retour avalé par la pause de focus ; un test du vrai runtime/UI reproduit ce défaut, puis vérifie la garde ciblée clavier/pointeur.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2328,12 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3e80c0f74e778afaec17e3eaf7ef381cf0d191473a04b0bff14552b74b254e2f</t>
+          <t xml:space="preserve">6ce9abe8fbe4a88b8fd10f438743bb05b9f31554f1f4b403b577b57656051924</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
@@ -2679,19 +2679,19 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2701,42 +2701,69 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4cd3effdc1e9f36ab7f64951288690ee93f910583dd448f920b9a6f35397875c</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
-      <c r="B31" s="0" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
-      <c r="C31" s="0" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
-      <c r="D31" s="0" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
-      <c r="E31" s="0" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
@@ -24422,7 +24449,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux cages et quatre ponts natifs ; approche continue sur sol624, fermeture et arrivée derrière les mêmes portes frontales156px Handoff de coordonnées délégué à useLift natif exclusivement pendant fermeture complète, même X et pieds ; cabine visible à ouverture Sauvegarde et reprise des quatre phases normales et du retour annulé ; contrôles exclusifs, annulation E pendant approche sans retour arrière et réouverture au pont source pendant trajet Sonde occupation destination pure : vrais corps owners et courtoisie sans reconstruire les PNJ hors champ Départ refusé si arrivée déjà occupée ; un blocage survenu pendant trajet ne peut plus piéger le joueur : E rouvre la cabine au pont source avant tout handoff</t>
+          <t xml:space="preserve">Deux cages et quatre ponts natifs ; approche continue sur sol624, fermeture et arrivée derrière les mêmes portes frontales156px Handoff de coordonnées délégué à useLift natif exclusivement pendant fermeture complète, même X et pieds ; cabine visible à ouverture Sauvegarde et reprise des quatre phases normales et du retour annulé ; contrôles exclusifs, annulation par clavier E ou bouton écran pendant approche et réouverture au pont source pendant trajet Sonde occupation destination pure : vrais corps owners et courtoisie sans reconstruire les PNJ hors champ Départ refusé si arrivée déjà occupée ; un blocage survenu pendant trajet ne peut plus piéger le joueur : E rouvre la cabine au pont source avant tout handoff</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -24566,17 +24593,17 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">27 nouvelles poses RGBA séparées pour les3cibles historiques, préparation Prowler à appuis conservés, chute articulée/maintien couché/contacts de deux corps/résistance/libération/récupération. Admission des15rigsV163 par leur catalogue source mesuré, liste historique4objets gardée. Aucun état de simulation modifié par le rendu. Raccord Prowler de la dernière prise réellement dessinée vers sa pose de libération en0,25s natif, sans rallonger le stun. Le segment de prise historique est masqué uniquement lorsque le nouvel atlas est réellement dessiné ; le HUD reste inchangé. L’ombre captive suit la racine visuelle et la largeur interpolée de la pose dessinée, séparément du corps de collision debout.</t>
+          <t xml:space="preserve">27 nouvelles poses RGBA séparées pour les3cibles historiques, préparation Prowler à appuis conservés, chute articulée/maintien couché/contacts de deux corps/résistance/libération/récupération. Admission des15rigsV163 par leur catalogue source mesuré, liste historique4objets gardée. Aucun état de simulation modifié par le rendu. Raccord Prowler de la dernière prise réellement dessinée vers sa pose de libération en0,25s natif, sans rallonger le stun. Correction de pause/reprise des prises natives : les commandes contrôlées directement conservent leur obligation de relâcher ; le CPU garde son entrée et sa progression de résistance après pause, sans prolongation de la prise ni modification du combat. La source du flux adverse est sérialisée, les anciens snapshots sans marqueur sont explicitement traités comme CPU et les changements direct/CPU restent bornés. Le HUD et son libellé accessible indiquent la garde pour un captif contrôlé directement, et la résistance adverse pour un captif CPU ; leurs lectures restent sans effet sur le combat. Le segment de prise historique est masqué uniquement lorsque le nouvel atlas est réellement dessiné ; le HUD reste inchangé. L’ombre captive suit la racine visuelle et la largeur interpolée de la pose dessinée, séparément du corps de collision debout.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js ; src/xeno-trials-capture-data-v163.js ; src/xeno-trials-runtime-v96.js ; src/xeno-trials-rig-v154.js ; src/xeno-trials-ui-v96.js ; src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js ; src/xeno-trials-capture-data-v163.js ; src/xeno-trials-runtime-v96.js ; src/xeno-trials-rig-v154.js ; src/xeno-trials-ui-v96.js ; src/xeno-trials-engine-v96.js ; src/xeno-trials-grapple-v153.js ; src/xeno-trials-grapple-v153.js</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/qa-xeno-trials-capture-v163.py</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/qa-xeno-trials-capture-v163.py</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
@@ -40661,7 +40688,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux cages et quatre ponts natifs ; approche continue sur sol624, fermeture et arrivée derrière les mêmes portes frontales156px Handoff de coordonnées délégué à useLift natif exclusivement pendant fermeture complète, même X et pieds ; cabine visible à ouverture Sauvegarde et reprise des quatre phases normales et du retour annulé ; contrôles exclusifs, annulation E pendant approche sans retour arrière et réouverture au pont source pendant trajet Sonde occupation destination pure : vrais corps owners et courtoisie sans reconstruire les PNJ hors champ Départ refusé si arrivée déjà occupée ; un blocage survenu pendant trajet ne peut plus piéger le joueur : E rouvre la cabine au pont source avant tout handoff</t>
+          <t xml:space="preserve">Deux cages et quatre ponts natifs ; approche continue sur sol624, fermeture et arrivée derrière les mêmes portes frontales156px Handoff de coordonnées délégué à useLift natif exclusivement pendant fermeture complète, même X et pieds ; cabine visible à ouverture Sauvegarde et reprise des quatre phases normales et du retour annulé ; contrôles exclusifs, annulation par clavier E ou bouton écran pendant approche et réouverture au pont source pendant trajet Sonde occupation destination pure : vrais corps owners et courtoisie sans reconstruire les PNJ hors champ Départ refusé si arrivée déjà occupée ; un blocage survenu pendant trajet ne peut plus piéger le joueur : E rouvre la cabine au pont source avant tout handoff</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -40737,12 +40764,12 @@
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js ; src/xeno-trials-capture-data-v163.js ; src/xeno-trials-runtime-v96.js ; src/xeno-trials-rig-v154.js ; src/xeno-trials-ui-v96.js ; src/xeno-trials-grapple-v153.js ; scripts/qa-xeno-trials-capture-v163.py</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js ; src/xeno-trials-capture-data-v163.js ; src/xeno-trials-runtime-v96.js ; src/xeno-trials-rig-v154.js ; src/xeno-trials-ui-v96.js ; src/xeno-trials-engine-v96.js ; src/xeno-trials-grapple-v153.js ; src/xeno-trials-grapple-v153.js ; scripts/qa-xeno-trials-capture-v163.py</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">27 nouvelles poses RGBA séparées pour les3cibles historiques, préparation Prowler à appuis conservés, chute articulée/maintien couché/contacts de deux corps/résistance/libération/récupération. Admission des15rigsV163 par leur catalogue source mesuré, liste historique4objets gardée. Aucun état de simulation modifié par le rendu. Raccord Prowler de la dernière prise réellement dessinée vers sa pose de libération en0,25s natif, sans rallonger le stun. Le segment de prise historique est masqué uniquement lorsque le nouvel atlas est réellement dessiné ; le HUD reste inchangé. L’ombre captive suit la racine visuelle et la largeur interpolée de la pose dessinée, séparément du corps de collision debout.</t>
+          <t xml:space="preserve">27 nouvelles poses RGBA séparées pour les3cibles historiques, préparation Prowler à appuis conservés, chute articulée/maintien couché/contacts de deux corps/résistance/libération/récupération. Admission des15rigsV163 par leur catalogue source mesuré, liste historique4objets gardée. Aucun état de simulation modifié par le rendu. Raccord Prowler de la dernière prise réellement dessinée vers sa pose de libération en0,25s natif, sans rallonger le stun. Correction de pause/reprise des prises natives : les commandes contrôlées directement conservent leur obligation de relâcher ; le CPU garde son entrée et sa progression de résistance après pause, sans prolongation de la prise ni modification du combat. La source du flux adverse est sérialisée, les anciens snapshots sans marqueur sont explicitement traités comme CPU et les changements direct/CPU restent bornés. Le HUD et son libellé accessible indiquent la garde pour un captif contrôlé directement, et la résistance adverse pour un captif CPU ; leurs lectures restent sans effet sur le combat. Le segment de prise historique est masqué uniquement lorsque le nouvel atlas est réellement dessiné ; le HUD reste inchangé. L’ombre captive suit la racine visuelle et la largeur interpolée de la pose dessinée, séparément du corps de collision debout.</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -41355,7 +41382,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/qa-xeno-trials-capture-v163.py</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/qa-xeno-trials-capture-v163.py</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix: keep compact motion tracker clear of elevated players
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -121,8 +121,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E32" totalsRowShown="0">
-  <autoFilter ref="A5:E32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E33" totalsRowShown="0">
+  <autoFilter ref="A5:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -2151,44 +2151,44 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
+          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
+          <t xml:space="preserve">src/npc-circulation-v158.js</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
+          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">806952ac6deaf7edb659c6f3c46254be7a569ac9a5b225e5b816a6e832a753cb</t>
+          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -2205,196 +2205,196 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e63cecc589a56bc2419eaf77a28fdba13279de78e1ad425567fd216a9981c09c</t>
+          <t xml:space="preserve">806952ac6deaf7edb659c6f3c46254be7a569ac9a5b225e5b816a6e832a753cb</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">205f5f27b47c9511964aedca4107bba4a388cc5bea791ae8348c818fe19d422c</t>
+          <t xml:space="preserve">e63cecc589a56bc2419eaf77a28fdba13279de78e1ad425567fd216a9981c09c</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">205f5f27b47c9511964aedca4107bba4a388cc5bea791ae8348c818fe19d422c</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requéraient une recette liée au candidat courant avec vrai parcours production/menu/Save. La preview production a ensuite reproduit un clic Retour avalé par la pause de focus ; un test du vrai runtime/UI reproduit ce défaut, puis vérifie la garde ciblée clavier/pointeur.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requéraient une recette liée au candidat courant avec vrai parcours production/menu/Save. La preview production a ensuite reproduit un clic Retour avalé par la pause de focus ; un test du vrai runtime/UI reproduit ce défaut, puis vérifie la garde ciblée clavier/pointeur.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sw.js</t>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c47b5a63287569005d7f01f04adf2db4658d5022e574471a77ab3d730c782b7</t>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">campaign-lethe-continuity-v163.css</t>
+          <t xml:space="preserve">sw.js</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">adac522847cbed1696f24a64f85d1c9c79cfa76b06088e812cca96e4dd2784ef</t>
+          <t xml:space="preserve">2c47b5a63287569005d7f01f04adf2db4658d5022e574471a77ab3d730c782b7</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
+          <t xml:space="preserve">campaign-lethe-continuity-v163.css</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
+          <t xml:space="preserve">adac522847cbed1696f24a64f85d1c9c79cfa76b06088e812cca96e4dd2784ef</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
+          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -2448,7 +2448,7 @@
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
+          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2485,24 +2485,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6ce9abe8fbe4a88b8fd10f438743bb05b9f31554f1f4b403b577b57656051924</t>
+          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2512,24 +2512,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">693127019ce88885f1a1a376016dda1910f82d45929431bd3acec0dce7fe95c6</t>
+          <t xml:space="preserve">6ce9abe8fbe4a88b8fd10f438743bb05b9f31554f1f4b403b577b57656051924</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">693127019ce88885f1a1a376016dda1910f82d45929431bd3acec0dce7fe95c6</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -2593,24 +2593,24 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2647,24 +2647,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
@@ -2691,7 +2691,7 @@
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -2718,7 +2718,7 @@
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -2745,25 +2745,52 @@
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
-      <c r="B32" s="0" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
-      <c r="D32" s="0" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
-      <c r="E32" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>

</xml_diff>

<commit_message>
fix: preserve crew collisions and readable mobile campaign flow
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -121,8 +121,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E33" totalsRowShown="0">
-  <autoFilter ref="A5:E33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E36" totalsRowShown="0">
+  <autoFilter ref="A5:E36"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -2070,287 +2070,287 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/app.js</t>
+          <t xml:space="preserve">mission-insertion-v62.css</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac0404430bb38a08b454bcc30a4d85a6af1f0afb57a953552739039cdc8180dd</t>
+          <t xml:space="preserve">192432c7cb0aad9d8b3d119cf5f819d031e92f27a8ad0eea8aab02dba2c532a2</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">74d0f90cefe5f9a5798795562bd348dc0695a840bfc5a9ed555e5f44d9c5285a</t>
+          <t xml:space="preserve">049525a19d40f882ce415330a1d467ebd26d7e3e641cffe76e19a61ecfeaffaf</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
+          <t xml:space="preserve">src/app.js</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
+          <t xml:space="preserve">ac0404430bb38a08b454bcc30a4d85a6af1f0afb57a953552739039cdc8180dd</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7112bc41d7952df2fc4affac5005613d7727041caba8ef5ec5a50e00aec70524</t>
+          <t xml:space="preserve">74d0f90cefe5f9a5798795562bd348dc0695a840bfc5a9ed555e5f44d9c5285a</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
+          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
+          <t xml:space="preserve">7112bc41d7952df2fc4affac5005613d7727041caba8ef5ec5a50e00aec70524</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
+          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette.</t>
+          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
+          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
+          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">806952ac6deaf7edb659c6f3c46254be7a569ac9a5b225e5b816a6e832a753cb</t>
+          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette.</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/npc-circulation-v158.js</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e63cecc589a56bc2419eaf77a28fdba13279de78e1ad425567fd216a9981c09c</t>
+          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">205f5f27b47c9511964aedca4107bba4a388cc5bea791ae8348c818fe19d422c</t>
+          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">806952ac6deaf7edb659c6f3c46254be7a569ac9a5b225e5b816a6e832a753cb</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requéraient une recette liée au candidat courant avec vrai parcours production/menu/Save. La preview production a ensuite reproduit un clic Retour avalé par la pause de focus ; un test du vrai runtime/UI reproduit ce défaut, puis vérifie la garde ciblée clavier/pointeur.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">e63cecc589a56bc2419eaf77a28fdba13279de78e1ad425567fd216a9981c09c</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">205f5f27b47c9511964aedca4107bba4a388cc5bea791ae8348c818fe19d422c</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -2367,115 +2367,115 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sw.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c47b5a63287569005d7f01f04adf2db4658d5022e574471a77ab3d730c782b7</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">campaign-lethe-continuity-v163.css</t>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">adac522847cbed1696f24a64f85d1c9c79cfa76b06088e812cca96e4dd2784ef</t>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
+          <t xml:space="preserve">sw.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
+          <t xml:space="preserve">2c47b5a63287569005d7f01f04adf2db4658d5022e574471a77ab3d730c782b7</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
+          <t xml:space="preserve">campaign-lethe-continuity-v163.css</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2485,12 +2485,12 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
+          <t xml:space="preserve">adac522847cbed1696f24a64f85d1c9c79cfa76b06088e812cca96e4dd2784ef</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC tout en conservant l’autorité du moteur natif et la compatibilité des sauvegardes.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -2502,7 +2502,7 @@
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2512,24 +2512,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6ce9abe8fbe4a88b8fd10f438743bb05b9f31554f1f4b403b577b57656051924</t>
+          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">693127019ce88885f1a1a376016dda1910f82d45929431bd3acec0dce7fe95c6</t>
+          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -2566,24 +2566,24 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -2593,24 +2593,24 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
+          <t xml:space="preserve">6ce9abe8fbe4a88b8fd10f438743bb05b9f31554f1f4b403b577b57656051924</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2620,24 +2620,24 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">ecf66b6474a9770a8d68d017659e623caca15965827c0330c28b9927f7f08d90</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2647,24 +2647,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2674,24 +2674,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2701,24 +2701,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2728,24 +2728,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
@@ -2772,25 +2772,106 @@
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
-      <c r="B33" s="0" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
-      <c r="C33" s="0" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
-      <c r="D33" s="0" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
-      <c r="E33" s="0" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
@@ -24380,17 +24461,17 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre chapitres originaux reliant les opérations natives QZ18, M577, C12 et Cocon Noir par un dossier et un ordre conseillé sans verrouillage supplémentaire. C12 et Cocon : cinq phases radio originales et deux choix de compte rendu chacun, avec pause/reprise et compatibilité des anciens checkpoints sans insertion. Première réussite native et dernier retour par chapitre, reçus bornés et états cohérents, données QZ/APC antérieures validées conservées, replis partiels distincts. Trois échanges explicitement lus par retour ; transaction atomique et sélection du plan existant sans paiement, lancement ni récompense automatiques.</t>
+          <t xml:space="preserve">Quatre chapitres originaux reliant les opérations natives QZ18, M577, C12 et Cocon Noir par un dossier et un ordre conseillé sans verrouillage supplémentaire. C12 et Cocon : cinq phases radio originales et deux choix de compte rendu chacun, avec pause/reprise et compatibilité des anciens checkpoints sans insertion. Première réussite native et dernier retour par chapitre, reçus bornés et états cohérents, données QZ/APC antérieures validées conservées, replis partiels distincts. Trois échanges explicitement lus par retour ; transaction atomique et sélection du plan existant sans paiement, lancement ni récompense automatiques. Insertion narrative lisible dans la largeur disponible : phase h2 adaptée au panneau, mise en page de lecture pleine largeur avec toolbar native et action PHOTOGRAPHIER dans le flux, hors du titre, et propriétaire de défilement vertical, uniquement tant que l’insertion est visible. La recette C12 reprise mesure root/parent/panneau/header/body, chaque bloc et ligne de dialogue, choix et actions aux viewports1600/390/320px ; elle conserve captures du composant et des vrais viewports et utilise la roulette native depuis le haut pour atteindre exactement les actions advance/pause, puis restaure le viewport avant le combat.</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-story-v163.js ; src/campaign-lethe-continuity-v163.js ; src/campaign-lethe-continuity-ui-v163.js ; campaign-lethe-continuity-v163.css</t>
+          <t xml:space="preserve">src/campaign-lethe-story-v163.js ; src/campaign-lethe-continuity-v163.js ; src/campaign-lethe-continuity-ui-v163.js ; campaign-lethe-continuity-v163.css ; mission-insertion-v62.css</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/qa-campaign-lethe-v163.py</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/qa-campaign-lethe-v163.py ; scripts/qa-campaign-story-v160.py ; scripts/qa-campaign-convoy-history-v162.py</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -24400,7 +24481,7 @@
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1.</t>
+          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1. Les contrôles de géométrie portent sur la préparation C12 réellement reprise ; ils ne certifient pas toutes les phases, toutes les campagnes ou une finition artistique globale. Les pilotes hérités conservent leurs assertions : les cinq identités V163 ne peuvent faire avancer que leur unique horloge d’animation finie et bornée au temps de rechargement mesuré.</t>
         </is>
       </c>
       <c r="I6" s="0">
@@ -24433,12 +24514,12 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js ; src/npc-service-traffic-v163.js ; src/npc-service-routes-v161.js ; src/npc-annex-leases-v163.js ; src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js ; src/npc-service-traffic-v163.js ; src/npc-service-routes-v161.js ; src/npc-annex-leases-v163.js ; src/npc-circulation-v158.js ; src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
@@ -24572,7 +24653,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote de vérification18parcours natifs :3presets livrés×3modes×desktop/mobile. Chargement des images, couches, visibilité des contrôles, clavier complet, retourOptions avecfocus/placement/angleetprofil exact conservés. Aucun correctif runtime hypothétique ou nouvel asset fabriqué.</t>
+          <t xml:space="preserve">Pilote de vérification18parcours natifs :3presets livrés×3modes×desktop/mobile. Chargement des images, couches, visibilité des contrôles, clavier complet, retourOptions avecfocus/placement/angleetprofil exact conservés. Aucun correctif runtime hypothétique ou nouvel asset fabriqué. Le contrat QA compare pour chaque mode les identifiants, rôles, rendus et images réellement définis dans le catalogue : Frontier compte 17/17/14 couches en full/reduced/static ; Storm et Ember 16/16/13. Les angles de vaisseau doivent appartenir aux assets orbitaux autorisés du preset.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -24592,7 +24673,7 @@
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1.</t>
+          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1. La comparaison QA conserve tous les changements de métadonnées réellement observés : seuls updatedAt et migratedFrom peuvent suivre le vrai commit du menu ; toutes les autres valeurs et leurs types restent strictement égaux. Aucun résultat d180 échoué n’est transféré. Les 18 parcours QA couvrent les trois presets existants sur deux viewports et trois modes ; les 21 combinaisons catalogue/angle/mode examinées séparément ne sont pas 21 nouveaux parcours natifs, décors ou assets.</t>
         </is>
       </c>
       <c r="I10" s="0">
@@ -24716,12 +24797,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote production unique démarrant par le vrai écran titre et le sélecteur de sauvegardes, avec profils initiaux explicitement déclarés. Broodstorm : lancement et six largages natifs, dont deux ratés ; sauvegarde du dernier projectile en vol, pause, rechargement du même profil, continuité balistique et impact ouvrant l’escorte, sans remboursement ni victoire inventée. Trials : trois duels production via le menu, règle publique 1 PV, verdicts CPU réels et quatre identités de sortie héritées. Pause exacte, coordonnées monde et caméra figées, redimensionnements 1280/1024/390 px, projection des marges hors canvas, fin bornée ou retour de navigation, conservation du reçu unique après rechargement. Captures séparées des pixels du vrai canvas et de son affichage CSS avec modale ; manifestes SHA des sources en début et fin de recette. Correction d’un défaut réel de navigation : le focus du bouton Retour ne peut plus ouvrir une modale qui intercepte son clic ou son activation clavier ; les commandes tenues sont libérées, les champs ordinaires et le blur conservent leur pause.</t>
+          <t xml:space="preserve">Pilote production unique démarrant par le vrai écran titre et le sélecteur de sauvegardes, avec profils initiaux explicitement déclarés. Broodstorm : lancement et six largages natifs, dont deux ratés ; sauvegarde du dernier projectile en vol, pause, rechargement du même profil, continuité balistique et impact ouvrant l’escorte, sans remboursement ni victoire inventée. Trials : trois duels production via le menu, règle publique 1 PV, verdicts CPU réels et quatre identités de sortie héritées. Pause exacte, coordonnées monde et caméra figées, redimensionnements 1280/1024/390 px, projection des marges hors canvas, fin bornée ou retour de navigation, conservation du reçu unique après rechargement. Captures séparées des pixels du vrai canvas et de son affichage CSS avec modale ; manifestes SHA des sources en début et fin de recette. Correction d’un défaut réel de navigation : le focus du bouton Retour ne peut plus ouvrir une modale qui intercepte son clic ou son activation clavier ; les commandes tenues sont libérées, les champs ordinaires et le blur conservent leur pause. Correction visuelle Broodstorm bornée à sa phase de vol : retirer le rectangle opaque de station36×48 qui recouvrait la navette Cheyenne, conserver ses pixels et le guidage label/E, couvrir l’ancien objectif dupliqué par un bandeau opaque102–202, et afficher la consigne utile CHARGES LIMITÉES. Les autres chapitres et les limites de l’adaptation dans le dossier/API sont conservés.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js ; src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -24736,7 +24817,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit.</t>
+          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit. Le correctif de rendu Broodstorm ne fournit aucun nouvel art ni chapitre complet ; il ne valide ni escorte, reine, extraction finale, ni fidélité franchise1:1. Les21tests ciblés du successeur partagé sont préliminaires ; seules de nouvelles captures natives liées au candidat exact peuvent vérifier le rendu corrigé. Aucun reçu d180 n’est transféré.</t>
         </is>
       </c>
       <c r="I13" s="0">
@@ -29299,7 +29380,7 @@
       </c>
       <c r="H82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1.</t>
+          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1. Les contrôles de géométrie portent sur la préparation C12 réellement reprise ; ils ne certifient pas toutes les phases, toutes les campagnes ou une finition artistique globale. Les pilotes hérités conservent leurs assertions : les cinq identités V163 ne peuvent faire avancer que leur unique horloge d’animation finie et bornée au temps de rechargement mesuré.</t>
         </is>
       </c>
       <c r="I82" s="0" t="inlineStr">
@@ -29589,7 +29670,7 @@
       </c>
       <c r="H87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les atlas dédiés NORMAL/SUCCESS/PERFECT/FAILED par famille restent absents. Un geste procédural corrigé n'est pas une nouvelle animation source dédiée. Les coordonnées service/grip existantes sont des mesures/tunings de silhouette du projet ; aucune certification canonique1:1. La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1.</t>
+          <t xml:space="preserve">Les atlas dédiés NORMAL/SUCCESS/PERFECT/FAILED par famille restent absents. Un geste procédural corrigé n'est pas une nouvelle animation source dédiée. Les coordonnées service/grip existantes sont des mesures/tunings de silhouette du projet ; aucune certification canonique1:1. La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1. La comparaison QA conserve tous les changements de métadonnées réellement observés : seuls updatedAt et migratedFrom peuvent suivre le vrai commit du menu ; toutes les autres valeurs et leurs types restent strictement égaux. Aucun résultat d180 échoué n’est transféré. Les 18 parcours QA couvrent les trois presets existants sur deux viewports et trois modes ; les 21 combinaisons catalogue/angle/mode examinées séparément ne sont pas 21 nouveaux parcours natifs, décors ou assets.</t>
         </is>
       </c>
       <c r="I87" s="0" t="inlineStr">
@@ -29705,7 +29786,7 @@
       </c>
       <c r="H89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit.</t>
+          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit. Le correctif de rendu Broodstorm ne fournit aucun nouvel art ni chapitre complet ; il ne valide ni escorte, reine, extraction finale, ni fidélité franchise1:1. Les21tests ciblés du successeur partagé sont préliminaires ; seules de nouvelles captures natives liées au candidat exact peuvent vérifier le rendu corrigé. Aucun reçu d180 n’est transféré.</t>
         </is>
       </c>
       <c r="I89" s="0" t="inlineStr">
@@ -29763,7 +29844,7 @@
       </c>
       <c r="H90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit.</t>
+          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit. Le correctif de rendu Broodstorm ne fournit aucun nouvel art ni chapitre complet ; il ne valide ni escorte, reine, extraction finale, ni fidélité franchise1:1. Les21tests ciblés du successeur partagé sont préliminaires ; seules de nouvelles captures natives liées au candidat exact peuvent vérifier le rendu corrigé. Aucun reçu d180 n’est transféré.</t>
         </is>
       </c>
       <c r="I90" s="0" t="inlineStr">
@@ -40656,17 +40737,17 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-story-v163.js ; src/campaign-lethe-continuity-v163.js ; src/campaign-lethe-continuity-ui-v163.js ; campaign-lethe-continuity-v163.css ; scripts/qa-campaign-lethe-v163.py</t>
+          <t xml:space="preserve">src/campaign-lethe-story-v163.js ; src/campaign-lethe-continuity-v163.js ; src/campaign-lethe-continuity-ui-v163.js ; campaign-lethe-continuity-v163.css ; mission-insertion-v62.css ; scripts/qa-campaign-lethe-v163.py ; scripts/qa-campaign-story-v160.py ; scripts/qa-campaign-convoy-history-v162.py</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre chapitres originaux reliant les opérations natives QZ18, M577, C12 et Cocon Noir par un dossier et un ordre conseillé sans verrouillage supplémentaire. C12 et Cocon : cinq phases radio originales et deux choix de compte rendu chacun, avec pause/reprise et compatibilité des anciens checkpoints sans insertion. Première réussite native et dernier retour par chapitre, reçus bornés et états cohérents, données QZ/APC antérieures validées conservées, replis partiels distincts. Trois échanges explicitement lus par retour ; transaction atomique et sélection du plan existant sans paiement, lancement ni récompense automatiques.</t>
+          <t xml:space="preserve">Quatre chapitres originaux reliant les opérations natives QZ18, M577, C12 et Cocon Noir par un dossier et un ordre conseillé sans verrouillage supplémentaire. C12 et Cocon : cinq phases radio originales et deux choix de compte rendu chacun, avec pause/reprise et compatibilité des anciens checkpoints sans insertion. Première réussite native et dernier retour par chapitre, reçus bornés et états cohérents, données QZ/APC antérieures validées conservées, replis partiels distincts. Trois échanges explicitement lus par retour ; transaction atomique et sélection du plan existant sans paiement, lancement ni récompense automatiques. Insertion narrative lisible dans la largeur disponible : phase h2 adaptée au panneau, mise en page de lecture pleine largeur avec toolbar native et action PHOTOGRAPHIER dans le flux, hors du titre, et propriétaire de défilement vertical, uniquement tant que l’insertion est visible. La recette C12 reprise mesure root/parent/panneau/header/body, chaque bloc et ligne de dialogue, choix et actions aux viewports1600/390/320px ; elle conserve captures du composant et des vrais viewports et utilise la roulette native depuis le haut pour atteindre exactement les actions advance/pause, puis restaure le viewport avant le combat.</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1.</t>
+          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1. Les contrôles de géométrie portent sur la préparation C12 réellement reprise ; ils ne certifient pas toutes les phases, toutes les campagnes ou une finition artistique globale. Les pilotes hérités conservent leurs assertions : les cinq identités V163 ne peuvent faire avancer que leur unique horloge d’animation finie et bornée au temps de rechargement mesuré.</t>
         </is>
       </c>
     </row>
@@ -40683,7 +40764,7 @@
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js ; src/npc-service-traffic-v163.js ; src/npc-service-routes-v161.js ; src/npc-annex-leases-v163.js ; src/npc-circulation-v158.js ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js ; src/npc-service-traffic-v163.js ; src/npc-service-routes-v161.js ; src/npc-annex-leases-v163.js ; src/npc-circulation-v158.js ; src/npc-life-v136.js ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
@@ -40769,12 +40850,12 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote de vérification18parcours natifs :3presets livrés×3modes×desktop/mobile. Chargement des images, couches, visibilité des contrôles, clavier complet, retourOptions avecfocus/placement/angleetprofil exact conservés. Aucun correctif runtime hypothétique ou nouvel asset fabriqué.</t>
+          <t xml:space="preserve">Pilote de vérification18parcours natifs :3presets livrés×3modes×desktop/mobile. Chargement des images, couches, visibilité des contrôles, clavier complet, retourOptions avecfocus/placement/angleetprofil exact conservés. Aucun correctif runtime hypothétique ou nouvel asset fabriqué. Le contrat QA compare pour chaque mode les identifiants, rôles, rendus et images réellement définis dans le catalogue : Frontier compte 17/17/14 couches en full/reduced/static ; Storm et Ember 16/16/13. Les angles de vaisseau doivent appartenir aux assets orbitaux autorisés du preset.</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1.</t>
+          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1. La comparaison QA conserve tous les changements de métadonnées réellement observés : seuls updatedAt et migratedFrom peuvent suivre le vrai commit du menu ; toutes les autres valeurs et leurs types restent strictement égaux. Aucun résultat d180 échoué n’est transféré. Les 18 parcours QA couvrent les trois presets existants sur deux viewports et trois modes ; les 21 combinaisons catalogue/angle/mode examinées séparément ne sont pas 21 nouveaux parcours natifs, décors ou assets.</t>
         </is>
       </c>
     </row>
@@ -40845,17 +40926,17 @@
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js ; scripts/qa-trials-continuity-v163.py</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js ; src/legacy-operations-v131.js ; scripts/qa-trials-continuity-v163.py</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote production unique démarrant par le vrai écran titre et le sélecteur de sauvegardes, avec profils initiaux explicitement déclarés. Broodstorm : lancement et six largages natifs, dont deux ratés ; sauvegarde du dernier projectile en vol, pause, rechargement du même profil, continuité balistique et impact ouvrant l’escorte, sans remboursement ni victoire inventée. Trials : trois duels production via le menu, règle publique 1 PV, verdicts CPU réels et quatre identités de sortie héritées. Pause exacte, coordonnées monde et caméra figées, redimensionnements 1280/1024/390 px, projection des marges hors canvas, fin bornée ou retour de navigation, conservation du reçu unique après rechargement. Captures séparées des pixels du vrai canvas et de son affichage CSS avec modale ; manifestes SHA des sources en début et fin de recette. Correction d’un défaut réel de navigation : le focus du bouton Retour ne peut plus ouvrir une modale qui intercepte son clic ou son activation clavier ; les commandes tenues sont libérées, les champs ordinaires et le blur conservent leur pause.</t>
+          <t xml:space="preserve">Pilote production unique démarrant par le vrai écran titre et le sélecteur de sauvegardes, avec profils initiaux explicitement déclarés. Broodstorm : lancement et six largages natifs, dont deux ratés ; sauvegarde du dernier projectile en vol, pause, rechargement du même profil, continuité balistique et impact ouvrant l’escorte, sans remboursement ni victoire inventée. Trials : trois duels production via le menu, règle publique 1 PV, verdicts CPU réels et quatre identités de sortie héritées. Pause exacte, coordonnées monde et caméra figées, redimensionnements 1280/1024/390 px, projection des marges hors canvas, fin bornée ou retour de navigation, conservation du reçu unique après rechargement. Captures séparées des pixels du vrai canvas et de son affichage CSS avec modale ; manifestes SHA des sources en début et fin de recette. Correction d’un défaut réel de navigation : le focus du bouton Retour ne peut plus ouvrir une modale qui intercepte son clic ou son activation clavier ; les commandes tenues sont libérées, les champs ordinaires et le blur conservent leur pause. Correction visuelle Broodstorm bornée à sa phase de vol : retirer le rectangle opaque de station36×48 qui recouvrait la navette Cheyenne, conserver ses pixels et le guidage label/E, couvrir l’ancien objectif dupliqué par un bandeau opaque102–202, et afficher la consigne utile CHARGES LIMITÉES. Les autres chapitres et les limites de l’adaptation dans le dossier/API sont conservés.</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit.</t>
+          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit. Le correctif de rendu Broodstorm ne fournit aucun nouvel art ni chapitre complet ; il ne valide ni escorte, reine, extraction finale, ni fidélité franchise1:1. Les21tests ciblés du successeur partagé sont préliminaires ; seules de nouvelles captures natives liées au candidat exact peuvent vérifier le rendu corrigé. Aucun reçu d180 n’est transféré.</t>
         </is>
       </c>
     </row>
@@ -41299,7 +41380,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/qa-campaign-lethe-v163.py</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/qa-campaign-lethe-v163.py ; scripts/qa-campaign-story-v160.py ; scripts/qa-campaign-convoy-history-v162.py</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -41309,7 +41390,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1.</t>
+          <t xml:space="preserve">Quatre opérations originales existantes : les455 entrées de campagnes du catalogue ne sont pas toutes des missions nouvelles entièrement validées par ce chantier. Aucune archive Blackout/Earth manquante ou scène filmique canonique n’est reconstruite ; fiction originale indiquée dans les données. Les scènes sont illustrées et radio, avec assets existants ; elles ne constituent pas des voix ou clips récupérés. Le pilote natif complète C12 ; il ne parcourt pas intégralement QZ18, APC ou toute la colonie/quarantaine Cocon dans sa propre session. Les anciens profils peuvent fournir un dossier QZ complet ou un historique APC validé : ils sont des reprises déclarées, jamais des parcours frais inventés. L’historique local est validé structurellement, pas signé cryptographiquement ; il n’autorise aucun paiement. La QA automatisée ne constitue pas une validation humaine ou 1:1. Les contrôles de géométrie portent sur la préparation C12 réellement reprise ; ils ne certifient pas toutes les phases, toutes les campagnes ou une finition artistique globale. Les pilotes hérités conservent leurs assertions : les cinq identités V163 ne peuvent faire avancer que leur unique horloge d’animation finie et bornée au temps de rechargement mesuré.</t>
         </is>
       </c>
     </row>
@@ -41321,7 +41402,7 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/qa-npc-annex-service-routes-v163.py ; scripts/qa-npc-annex-leases-v163.py</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -41397,7 +41478,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1.</t>
+          <t xml:space="preserve">La demande historique de20presets artistiques dédiés reste ouverte :17autres décors planétaires/35slots historiques absents. V79/V87/V90 existants sont déjà branchés. Les variantes de présentation ne sont pas20nouvelles compositions artistiques. Pas de nouvelle composition titre livrée ni certification artistique1:1. La comparaison QA conserve tous les changements de métadonnées réellement observés : seuls updatedAt et migratedFrom peuvent suivre le vrai commit du menu ; toutes les autres valeurs et leurs types restent strictement égaux. Aucun résultat d180 échoué n’est transféré. Les 18 parcours QA couvrent les trois presets existants sur deux viewports et trois modes ; les 21 combinaisons catalogue/angle/mode examinées séparément ne sont pas 21 nouveaux parcours natifs, décors ou assets.</t>
         </is>
       </c>
     </row>
@@ -41463,7 +41544,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit.</t>
+          <t xml:space="preserve">Couverture automatisée de continuité ; aucune validation humaine ni certification canonique1:1. Broodstorm s’arrête à la destruction réelle du second nid par la dernière bombe restaurée ; escorte, reine et extraction finale ne sont pas revendiquées par ce pilote. Le profil Trials déclare quatre déblocages initiaux non gagnés ; la règle 1 PV est sélectionnée dans l’interface existante, sans écriture de santé dans le moteur. Les quatre identités de sortie héritées sont couvertes ; nouveaux dessins, audio, tours de dos, locomotion entièrement dessinée et autres identités restent ouverts. Les projections CSS vérifient la géométrie du viewport ; les captures conservent les pixels natifs réellement observés. Aucun visuel de film ou résultat de combat n’est reconstruit. Le correctif de rendu Broodstorm ne fournit aucun nouvel art ni chapitre complet ; il ne valide ni escorte, reine, extraction finale, ni fidélité franchise1:1. Les21tests ciblés du successeur partagé sont préliminaires ; seules de nouvelles captures natives liées au candidat exact peuvent vérifier le rendu corrigé. Aucun reçu d180 n’est transféré.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix reviewed opaque NPC pockets in world sprites and dialogue portraits
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -121,8 +121,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E36" totalsRowShown="0">
-  <autoFilter ref="A5:E36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E39" totalsRowShown="0">
+  <autoFilter ref="A5:E39"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -2107,17 +2107,17 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">74d0f90cefe5f9a5798795562bd348dc0695a840bfc5a9ed555e5f44d9c5285a</t>
+          <t xml:space="preserve">418385128f0a42d5df8d793fc775424ff6cd4153f94466a02e65f6297fcdae98</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique.</t>
+          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique. Appliquer aussi aux portraits natifs le masque V164 des seules poches de fond admises, en conservant les PNG et le cadrage et en retirant le masque lors de chaque changement de source.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2610,7 @@
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2620,24 +2620,24 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ecf66b6474a9770a8d68d017659e623caca15965827c0330c28b9927f7f08d90</t>
+          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
+          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">ecf66b6474a9770a8d68d017659e623caca15965827c0330c28b9927f7f08d90</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -2664,7 +2664,7 @@
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
@@ -2691,7 +2691,7 @@
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2701,24 +2701,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">16e7eb2bc96f16c7f404748463d7374e5d5fcc7fa46ec9d73b966b41c24c0e6f</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">Épingler les sources et runs exacts de vingt-quatre poches de fond dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2728,24 +2728,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">5b27f25b90688989c4d3ba0627ae746f1c155b2f5a1b01aef50b072b4d725324</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
+          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2755,24 +2755,24 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">cd4b19be365797e185bd6d55e4125457decc134e4298dfd4a18a544b9a7ca3b2</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker.</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2782,24 +2782,24 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -2809,24 +2809,24 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction.</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
@@ -2853,25 +2853,106 @@
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur.</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
-      <c r="B36" s="0" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
-      <c r="C36" s="0" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
-      <c r="D36" s="0" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence.</t>
         </is>
       </c>
-      <c r="E36" s="0" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
@@ -27345,7 +27426,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -27403,7 +27484,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -27461,7 +27542,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -27519,7 +27600,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -27577,7 +27658,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -27635,7 +27716,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -27751,7 +27832,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -27809,7 +27890,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -27867,7 +27948,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -27925,7 +28006,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -27983,7 +28064,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -28041,7 +28122,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -28157,7 +28238,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -28215,7 +28296,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -28273,7 +28354,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -28331,7 +28412,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -28389,7 +28470,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -28447,7 +28528,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -28563,7 +28644,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -28621,7 +28702,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -28679,7 +28760,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -28737,7 +28818,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TECHNIQUE_V163_IMPLEMENTEE_RECETTE_ROOT_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -28795,7 +28876,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -28853,7 +28934,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERITAGE_ET_EXTENSION_V163_A_REVERIFIER_SUR_RECETTE_ROOT</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -28911,17 +28992,17 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RECETTE_EXACTE_V163_NON_EXECUTEE</t>
+          <t xml:space="preserve">MERGED_EXACT_TESTED_TREE</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aucun résultat préliminaire ni historique ne constitue une recette complète du candidat final V163.</t>
+          <t xml:space="preserve">Conserver ces reçus comme historique du lot ; toute évolution ultérieure exige sa propre recette.</t>
         </is>
       </c>
       <c r="I74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Figer le candidat propre, exécuter toutes les recettes déclarées, conserver les reçus puis constater la CI et la fusion du même arbre.</t>
+          <t xml:space="preserve">Conserver les reçus du lot ; une évolution ultérieure exige sa propre recette.</t>
         </is>
       </c>
       <c r="J74" s="0" t="inlineStr">
@@ -29027,7 +29108,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -29143,7 +29224,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -29201,7 +29282,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -29375,7 +29456,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -29491,7 +29572,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -29665,7 +29746,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -29723,7 +29804,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -29781,7 +29862,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -29839,7 +29920,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PERIMETRE_V163_LIVRE_OU_RECETTE_PREPAREE_PREUVES_EXACTES_PENDING</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -29957,7 +30038,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -30143,7 +30224,7 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_NATIF_HERITE_QA_V163_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -30701,7 +30782,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -30732,7 +30813,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -30763,7 +30844,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -30794,7 +30875,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
@@ -30825,7 +30906,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -30856,7 +30937,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -33646,7 +33727,7 @@
       </c>
       <c r="D125" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E125" s="0" t="inlineStr">
@@ -33956,7 +34037,7 @@
       </c>
       <c r="D135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E135" s="0" t="inlineStr">
@@ -34080,7 +34161,7 @@
       </c>
       <c r="D139" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E139" s="0" t="inlineStr">
@@ -34390,7 +34471,7 @@
       </c>
       <c r="D149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_NATIF_HERITE_QA_V163_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E149" s="0" t="inlineStr">
@@ -34514,7 +34595,7 @@
       </c>
       <c r="D153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_NATIF_HERITE_QA_V163_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E153" s="0" t="inlineStr">
@@ -34886,7 +34967,7 @@
       </c>
       <c r="D165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E165" s="0" t="inlineStr">
@@ -34979,7 +35060,7 @@
       </c>
       <c r="D168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_NATIF_HERITE_QA_V163_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E168" s="0" t="inlineStr">
@@ -35103,7 +35184,7 @@
       </c>
       <c r="D172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E172" s="0" t="inlineStr">
@@ -35320,7 +35401,7 @@
       </c>
       <c r="D179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E179" s="0" t="inlineStr">
@@ -35351,7 +35432,7 @@
       </c>
       <c r="D180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E180" s="0" t="inlineStr">
@@ -35382,7 +35463,7 @@
       </c>
       <c r="D181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIG_PRESENTATION_V163_VERIFICATEUR_CIBLE_RECETTE_VISUELLE_A_EXECUTER</t>
+          <t xml:space="preserve">PASSED_EXACT_HEAD_WITH_DECLARED_LIMITS</t>
         </is>
       </c>
       <c r="E181" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Include NPC matte modules in the verified offline shell
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -2458,17 +2458,17 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c47b5a63287569005d7f01f04adf2db4658d5022e574471a77ab3d730c782b7</t>
+          <t xml:space="preserve">cb6eb87ee7f5b25bc822f6fbaf035128497c10876aa72c6b879e7fbec0a32994</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées.</t>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
+          <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete confirmed NPC masks and preserve exact release evidence
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -547,10 +547,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -919,6 +919,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
 </worksheet>
 </file>
 
@@ -946,10 +949,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -1206,6 +1209,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -1238,10 +1244,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -1976,6 +1982,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2006,10 +2015,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -2458,17 +2467,17 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cb6eb87ee7f5b25bc822f6fbaf035128497c10876aa72c6b879e7fbec0a32994</t>
+          <t xml:space="preserve">428232e7d31e03925f3ca9d60c6980a47fc3cbd73acc2d72d1430b1e0a151ea6</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution.</t>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs</t>
+          <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
       </c>
     </row>
@@ -2701,12 +2710,12 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">16e7eb2bc96f16c7f404748463d7374e5d5fcc7fa46ec9d73b966b41c24c0e6f</t>
+          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler les sources et runs exacts de vingt-quatre poches de fond dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses.</t>
+          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -2728,7 +2737,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5b27f25b90688989c4d3ba0627ae746f1c155b2f5a1b01aef50b072b4d725324</t>
+          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -2959,6 +2968,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2992,10 +3004,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -3194,6 +3206,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -3231,10 +3246,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -10893,6 +10908,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:L3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -10927,10 +10945,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -14037,6 +14055,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:I3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -14069,10 +14090,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -14151,6 +14172,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -14187,10 +14211,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -15047,6 +15071,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:K3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -15085,10 +15112,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -20976,6 +21003,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:M3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -21014,10 +21044,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -21341,6 +21371,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:M3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -21374,10 +21407,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -22944,6 +22977,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -22982,10 +23018,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -23687,6 +23723,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:M3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -23719,10 +23758,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -23904,6 +23943,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -23939,10 +23981,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -24143,6 +24185,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:J3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -24178,10 +24223,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -24430,6 +24475,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:J3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -24465,10 +24513,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -24909,6 +24957,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:J3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -24946,10 +24997,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -29946,6 +29997,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:L3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -29978,10 +30032,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -35882,6 +35936,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -35915,10 +35972,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -37085,6 +37142,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -37118,10 +37178,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -38688,6 +38748,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -38721,10 +38784,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -39569,6 +39632,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -39599,10 +39665,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -39958,6 +40024,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -39988,10 +40057,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -41373,6 +41442,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -41402,10 +41474,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -41444,7 +41516,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -41466,7 +41538,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
@@ -41488,7 +41560,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -41510,7 +41582,7 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -41532,7 +41604,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -41554,7 +41626,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -41576,7 +41648,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -41598,7 +41670,7 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -41620,7 +41692,7 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
@@ -41642,7 +41714,7 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À exécuter sur le commit final</t>
+          <t xml:space="preserve">V164 : à exécuter sur son propre commit</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -41664,7 +41736,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">À vérifier séparément</t>
+          <t xml:space="preserve">V164 : à vérifier, CI, revue et fusion propres</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -41674,6 +41746,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:D3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -41705,10 +41780,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prépublication : implémentation et validation du commit restent distinctes.</t>
+          <t xml:space="preserve">Livraison V163 : 043bb60 vers 8a934b7 ; 2 993 tests, 16 profils, 1 566 contrôles, 835 PNG. Contrats maintenus pour V164 : nouvelle validation requise.</t>
         </is>
       </c>
     </row>
@@ -46659,6 +46734,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:F3"/>
+  </mergeCells>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
docs: pin station relay sources and preserve open validation scope
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -122,8 +122,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E67" totalsRowShown="0">
-  <autoFilter ref="A5:E67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E68" totalsRowShown="0">
+  <autoFilter ref="A5:E68"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V162"/>
@@ -2162,17 +2162,17 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">640bfebbf1e4df8e214f4126065e9dc3ddd77714e28e0444dbb4dfc227bea55c</t>
+          <t xml:space="preserve">52df812dec93254e16133812240e2bf511df4f90a231661f511502868a8b9803</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique. Appliquer aussi aux portraits natifs le masque V164 des seules poches de fond admises, en conservant les PNG et le cadrage et en retirant le masque lors de chaque changement de source. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures.</t>
+          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique. Appliquer aussi aux portraits natifs le masque V164 des seules poches de fond admises, en conservant les PNG et le cadrage et en retirant le masque lors de chaque changement de source. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-npc-matte-apertures-v164.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-npc-matte-apertures-v164.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2405,17 +2405,17 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d31e6ca7367b2453f846f46f09afc883d9e99500796ae7ff53f90d95ce4038a</t>
+          <t xml:space="preserve">05c6efb9553eb7908a633b1c811651efe6c292c4a036c2f8628fa051c1bae824</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2626,12 +2626,12 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2680,12 +2680,12 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2707,12 +2707,12 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2734,12 +2734,12 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2788,12 +2788,12 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2815,12 +2815,12 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2891,17 +2891,17 @@
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cc77869c8b7b1a190b7e245dee7cd4ad3f5f77fafc4cc76f50132118b65f428f</t>
+          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2977,12 +2977,12 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -2999,17 +2999,17 @@
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">366937c0857cfa04fdf4126a8127eeb7244630a59b1cf83e96c1b0342475f821</t>
+          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
@@ -3026,61 +3026,61 @@
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">03295bc1ce6bafcc21df538804fb3fa492c34da82f997e56ba8cc17fe60242af</t>
+          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
+          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
+          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
+          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
@@ -3097,17 +3097,17 @@
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
+          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
@@ -3124,34 +3124,34 @@
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
+          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
+          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
@@ -3178,7 +3178,7 @@
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
+          <t xml:space="preserve">src/player-appearance-v126.js</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
+          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
@@ -3205,7 +3205,7 @@
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
+          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
+          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -3232,7 +3232,7 @@
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
+          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
+          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -3259,44 +3259,44 @@
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
+          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
+          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
@@ -3313,17 +3313,17 @@
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">63e7894684e439701fbccca1f61a0cdea5e021ff80c2d3e4bd5fc7bd1a452c6b</t>
+          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
@@ -3340,34 +3340,34 @@
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
+          <t xml:space="preserve">63e7894684e439701fbccca1f61a0cdea5e021ff80c2d3e4bd5fc7bd1a452c6b</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/refuge-art-v87.js</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
@@ -3377,78 +3377,78 @@
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes.</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cef500ca64bd66b4aa5e933a2f0794d88fbe197405f61fd95bb7e27f8e0bba89</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
@@ -3458,24 +3458,24 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
@@ -3502,7 +3502,7 @@
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
@@ -3529,7 +3529,7 @@
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -3556,7 +3556,7 @@
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
@@ -3566,24 +3566,24 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
@@ -3593,150 +3593,177 @@
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
         </is>
       </c>
     </row>
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="48" customHeight="1">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B67" s="0" t="inlineStr">
+      <c r="B68" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
-      <c r="C67" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">592bb81be5f5152e6bf74fe817d7f671cd41d43e5777153fd3cf1c3a0aea1078</t>
-        </is>
-      </c>
-      <c r="D67" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge.</t>
-        </is>
-      </c>
-      <c r="E67" s="0" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08b0a5d0e44e988f05e0730c404befd654f20e03052ceeaf53d256cabf6b5500</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165.</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
@@ -25445,22 +25472,22 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deux boucles locales Rook/CCTV et Tamsin/range ; Cal vers le vrai catwalk logistique ; quatre services inter-ponts David, Inez, Maksim et Jun en construction.</t>
+          <t xml:space="preserve">Deux services locaux Rook/CCTV et Tamsin/range complétés en V166 par leurs départs et retours physiques depuis capteurs et briefing, avec cabines partagées ; Cal vers le vrai catwalk logistique ; quatre services inter-ponts David, Inez, Maksim et Jun.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aucune clôture des sept trajets ou de leurs voyages complets déduite de la présence des contrôleurs. Origines de poste locales distinctes des stations lointaines ; portions macro non observées signalées.</t>
+          <t xml:space="preserve">Les trajets V166 sont couverts par vingt scénarios de service et cinq de portes ; leur pilote navigateur reste à exécuter. Aucune clôture des sept trajets ou validation humaine déduite du code ou des tests. Les reçus V165 antérieurs ne valident pas ce candidat.</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js ; src/npc-cal-logistics-route-v165.js ; src/npc-interdeck-routes-v165.js ; src/npc-interdeck-passage-v165.js ; src/npc-lift-transit-v165.js ; src/npc-cal-climb-rig-v165.js ; src/npc-jun-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js ; src/npc-cal-logistics-route-v165.js ; src/npc-interdeck-routes-v165.js ; src/npc-interdeck-passage-v165.js ; src/npc-lift-transit-v165.js ; src/npc-cal-climb-rig-v165.js ; src/npc-jun-climb-rig-v165.js ; src/npc-station-relays-v166.js</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/qa-npc-annex-workpost-routes-v165.py ; scripts/qa-npc-cal-logistics-route-v165.py ; scripts/qa-npc-interdeck-native-v165.py ; scripts/qa-npc-interdeck-routes-v165.py</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs ; scripts/qa-npc-annex-workpost-routes-v165.py ; scripts/qa-npc-cal-logistics-route-v165.py ; scripts/qa-npc-interdeck-native-v165.py ; scripts/qa-npc-interdeck-routes-v165.py ; scripts/qa-npc-station-relays-v166.py</t>
         </is>
       </c>
       <c r="H8" s="0">

</xml_diff>

<commit_message>
fix: synchronize human gait and mount Tantalus door signs
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -122,8 +122,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E68" totalsRowShown="0">
-  <autoFilter ref="A5:E68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E70" totalsRowShown="0">
+  <autoFilter ref="A5:E70"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V162"/>
@@ -2329,12 +2329,12 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-game.js</t>
+          <t xml:space="preserve">src/hub-bulkhead-depth-v134.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -2378,24 +2378,24 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e6c4101e04579252bc6045e22cb9305921fbe20c931072732d9a9e045e15b3e</t>
+          <t xml:space="preserve">b330fdbf92aa34f8cfb49b58a9229bdedbf4a17ec11663d9ae6e2146a1eec41b</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : protéger les champs de saisie et consommer la touche native d’interaction avant l’ouverture et le focus synchrones du dialogue du refuge, afin que son action clavier par défaut ne rajoute pas un e au nom relu ; conserver les autres contrôles du moteur.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-interaction-input-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
+          <t xml:space="preserve">src/hub-game.js</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -2405,78 +2405,78 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">05c6efb9553eb7908a633b1c811651efe6c292c4a036c2f8628fa051c1bae824</t>
+          <t xml:space="preserve">2e6c4101e04579252bc6045e22cb9305921fbe20c931072732d9a9e045e15b3e</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : protéger les champs de saisie et consommer la touche native d’interaction avant l’ouverture et le focus synchrones du dialogue du refuge, afin que son action clavier par défaut ne rajoute pas un e au nom relu ; conserver les autres contrôles du moteur.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-interaction-input-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-life-v136.js</t>
+          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ee7433e6b7d663d4c4cee0da5a366617b0141cafad0a63e0928e4924e3b6b7f3</t>
+          <t xml:space="preserve">05c6efb9553eb7908a633b1c811651efe6c292c4a036c2f8628fa051c1bae824</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-service-details-v165.js</t>
+          <t xml:space="preserve">src/hub-room-life-v136.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b6eb5e20ca9c221399135afa5b5fc48d471df74daf9625c194fefe16099037b2</t>
+          <t xml:space="preserve">ee7433e6b7d663d4c4cee0da5a366617b0141cafad0a63e0928e4924e3b6b7f3</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
+          <t xml:space="preserve">src/hub-room-service-details-v165.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -2486,24 +2486,24 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d1ebb86dcebb09f6f586711ed3c7c2da7ab3909d609cdc1649549d5f592ecd25</t>
+          <t xml:space="preserve">b6eb5e20ca9c221399135afa5b5fc48d471df74daf9625c194fefe16099037b2</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
+          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2513,132 +2513,132 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
+          <t xml:space="preserve">5c9283b4f848a9a5882809f7b4f3c8c84478ed756f89bdc329cd1b875e8e0fe6</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/legacy-operations-v131.js</t>
+          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
+          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
+          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
+          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
+          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
+          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
+          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
+          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2648,24 +2648,24 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2675,24 +2675,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
+          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
@@ -2719,7 +2719,7 @@
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
+          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
+          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -2746,61 +2746,61 @@
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
+          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
+          <t xml:space="preserve">src/npc-circulation-v158.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
+          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
+          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccaad4fde98950522f516b7a33aba94de5bff169027985b567b7c2a9804fa9f1</t>
+          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
+          <t xml:space="preserve">ccaad4fde98950522f516b7a33aba94de5bff169027985b567b7c2a9804fa9f1</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
@@ -2854,61 +2854,61 @@
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-life-v136.js</t>
+          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
+          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
+          <t xml:space="preserve">src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
+          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
+          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
@@ -2918,24 +2918,24 @@
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
+          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
+          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
@@ -2945,12 +2945,12 @@
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
+          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
+          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -2962,7 +2962,7 @@
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
+          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
@@ -2972,61 +2972,61 @@
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
+          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
+          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
+          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="41" ht="48" customHeight="1">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
+          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
@@ -3043,7 +3043,7 @@
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
@@ -3053,132 +3053,132 @@
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
+          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
+          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
+          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
+          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
+          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
+          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
+          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
@@ -3205,7 +3205,7 @@
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
+          <t xml:space="preserve">src/player-appearance-v126.js</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
+          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -3232,7 +3232,7 @@
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
+          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
+          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -3259,7 +3259,7 @@
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
+          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
+          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
@@ -3286,115 +3286,115 @@
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
+          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
+          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">63e7894684e439701fbccca1f61a0cdea5e021ff80c2d3e4bd5fc7bd1a452c6b</t>
+          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
+          <t xml:space="preserve">2fef117a684b16b6c426ed93f932ce91e660648682f50600c799f5cd6126c8f9</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/refuge-art-v87.js</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
@@ -3404,78 +3404,78 @@
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
@@ -3485,24 +3485,24 @@
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
@@ -3512,24 +3512,24 @@
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -3556,7 +3556,7 @@
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
@@ -3583,7 +3583,7 @@
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
@@ -3593,24 +3593,24 @@
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
@@ -3620,150 +3620,204 @@
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
         </is>
       </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="48" customHeight="1">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="48" customHeight="1">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B68" s="0" t="inlineStr">
+      <c r="B70" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
-      <c r="C68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08b0a5d0e44e988f05e0730c404befd654f20e03052ceeaf53d256cabf6b5500</t>
-        </is>
-      </c>
-      <c r="D68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165.</t>
-        </is>
-      </c>
-      <c r="E68" s="0" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f51ae4141ecbf889dfd79261f0442d46f8b5b837e0038f8e8291ad157c604e6b</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165. Suite V167 : nouveau cache des mouvements humains et plaques de portes.</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
@@ -25558,7 +25612,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Révision des appuis et attaches du bassin, des jambes et du torse ; cadence liée à la distance, continuité marche/arrêt et présentation des humains alliés.</t>
+          <t xml:space="preserve">Révision des appuis et attaches du bassin, des jambes et du torse ; cadence liée à la distance, continuité marche/arrêt et présentation des humains alliés. Suite V167 : bras mains libres synchronisés aux pas ; continuité des alliés à travers les actions et rejet des faux pas sans temps écoulé.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -25568,12 +25622,12 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/human-patrol-animation-v133.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/human-patrol-animation-v133.js ; src/sprite-animation-runtime.js</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/qa-player-allies-contacts-v165.py</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/qa-player-allies-contacts-v165.py</t>
         </is>
       </c>
       <c r="H10" s="0">
@@ -25601,7 +25655,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 assemblages de service pour 35 profils de pièces ; quatre vues volontairement dégagées. Plaque du vrai nom sur le cadre du refuge ; retrait des gros libellés de développement.</t>
+          <t xml:space="preserve">31 assemblages de service pour 35 profils de pièces ; quatre vues volontairement dégagées. Plaque du vrai nom sur le cadre du refuge ; retrait des gros libellés de développement. Suite V167 : plaques physiques de destination fixées aux douze linteaux, dans les deux projections.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -25611,12 +25665,12 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-service-details-v165.js ; src/hub-room-life-v136.js ; src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/hub-room-service-details-v165.js ; src/hub-room-life-v136.js ; src/refuge-art-v87.js ; src/hub-bulkhead-depth-v134.js</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/qa-hub-service-details-v165.py</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/qa-hub-service-details-v165.py</t>
         </is>
       </c>
       <c r="H11" s="0">

</xml_diff>

<commit_message>
fix: preserve observed NPC stations and restore range crew dialogue
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -122,8 +122,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E70" totalsRowShown="0">
-  <autoFilter ref="A5:E70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E71" totalsRowShown="0">
+  <autoFilter ref="A5:E71"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V162"/>
@@ -2383,12 +2383,12 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
         </is>
       </c>
     </row>
@@ -2491,19 +2491,19 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
+          <t xml:space="preserve">src/hub-v81-runtime.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2513,24 +2513,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5c9283b4f848a9a5882809f7b4f3c8c84478ed756f89bdc329cd1b875e8e0fe6</t>
+          <t xml:space="preserve">26a75cc4fe0e7280146b370c9183cd89a52dabddd865f408289439fe824e4067</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
+          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2540,132 +2540,132 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
+          <t xml:space="preserve">5c9283b4f848a9a5882809f7b4f3c8c84478ed756f89bdc329cd1b875e8e0fe6</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/legacy-operations-v131.js</t>
+          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
+          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
+          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
+          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
+          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
+          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
+          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
+          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2675,24 +2675,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2702,24 +2702,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
+          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
+          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2756,12 +2756,12 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
+          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -2773,61 +2773,61 @@
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
+          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
+          <t xml:space="preserve">src/npc-circulation-v158.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
+          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
+          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -2837,12 +2837,12 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccaad4fde98950522f516b7a33aba94de5bff169027985b567b7c2a9804fa9f1</t>
+          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -2864,12 +2864,12 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
+          <t xml:space="preserve">85a4805f83ddaee04d830a80ca070d3903d7f5933720f859ffd5f7ca489f77c1</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -2881,61 +2881,61 @@
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-life-v136.js</t>
+          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
+          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
+          <t xml:space="preserve">src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
+          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
+          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
@@ -2945,24 +2945,24 @@
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
+          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
+          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
@@ -2972,12 +2972,12 @@
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
+          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
+          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -2989,7 +2989,7 @@
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
+          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
@@ -2999,66 +2999,66 @@
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
+          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="41" ht="48" customHeight="1">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
+          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
+          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
+          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -3070,7 +3070,7 @@
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
@@ -3080,61 +3080,61 @@
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
+          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
+          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
+          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
+          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
@@ -3151,17 +3151,17 @@
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
+          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
@@ -3178,34 +3178,34 @@
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
+          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
+          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -3232,7 +3232,7 @@
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
+          <t xml:space="preserve">src/player-appearance-v126.js</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
+          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -3259,7 +3259,7 @@
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
+          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
+          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
@@ -3286,7 +3286,7 @@
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
+          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
+          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
@@ -3313,44 +3313,44 @@
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
+          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
+          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
@@ -3367,17 +3367,17 @@
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2fef117a684b16b6c426ed93f932ce91e660648682f50600c799f5cd6126c8f9</t>
+          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
@@ -3394,34 +3394,34 @@
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
+          <t xml:space="preserve">2fef117a684b16b6c426ed93f932ce91e660648682f50600c799f5cd6126c8f9</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/refuge-art-v87.js</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
@@ -3431,78 +3431,78 @@
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
+          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
@@ -3512,24 +3512,24 @@
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
         </is>
       </c>
     </row>
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
@@ -3539,24 +3539,24 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
@@ -3583,7 +3583,7 @@
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
@@ -3610,7 +3610,7 @@
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
@@ -3637,7 +3637,7 @@
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
@@ -3647,24 +3647,24 @@
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
@@ -3674,150 +3674,177 @@
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
         </is>
       </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="48" customHeight="1">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B70" s="0" t="inlineStr">
+      <c r="B71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
-      <c r="C70" s="0" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">f51ae4141ecbf889dfd79261f0442d46f8b5b837e0038f8e8291ad157c604e6b</t>
         </is>
       </c>
-      <c r="D70" s="0" t="inlineStr">
+      <c r="D71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165. Suite V167 : nouveau cache des mouvements humains et plaques de portes.</t>
         </is>
       </c>
-      <c r="E70" s="0" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
@@ -25670,7 +25697,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/qa-hub-service-details-v165.py</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/qa-hub-service-details-v165.py</t>
         </is>
       </c>
       <c r="H11" s="0">

</xml_diff>

<commit_message>
feat: frame speaker avatars and furnish the Tantalus with batch100
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -122,8 +122,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E71" totalsRowShown="0">
-  <autoFilter ref="A5:E71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E80" totalsRowShown="0">
+  <autoFilter ref="A5:E80"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V162"/>
@@ -2098,115 +2098,115 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">index.html</t>
+          <t xml:space="preserve">hub-stations-v61.css</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9cce9373641e8440201bf6d64cd5b48ae0dfcab7f7cc90c5fe6230e9d2c500e0</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a4f5bf1470b0b736451ffbb74cc7c07994d2c9a6f9816bb9e81f53016253d6f5</t>
+          <t xml:space="preserve">eaf2b041ec39337b763d6d919859a7f79276c5eff920049980428b365202dfd5</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charger les styles et contrats de présentation livrés avec la continuité de campagne et maintenir leur intégration effective dans le document de production. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">mission-insertion-v62.css</t>
+          <t xml:space="preserve">index.html</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">192432c7cb0aad9d8b3d119cf5f819d031e92f27a8ad0eea8aab02dba2c532a2</t>
+          <t xml:space="preserve">9cce9373641e8440201bf6d64cd5b48ae0dfcab7f7cc90c5fe6230e9d2c500e0</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">049525a19d40f882ce415330a1d467ebd26d7e3e641cffe76e19a61ecfeaffaf</t>
+          <t xml:space="preserve">a4f5bf1470b0b736451ffbb74cc7c07994d2c9a6f9816bb9e81f53016253d6f5</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement. </t>
+          <t xml:space="preserve">Charger les styles et contrats de présentation livrés avec la continuité de campagne et maintenir leur intégration effective dans le document de production. </t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-public-release-v86.mjs</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/app.js</t>
+          <t xml:space="preserve">mission-insertion-v62.css</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac0404430bb38a08b454bcc30a4d85a6af1f0afb57a953552739039cdc8180dd</t>
+          <t xml:space="preserve">192432c7cb0aad9d8b3d119cf5f819d031e92f27a8ad0eea8aab02dba2c532a2</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">52df812dec93254e16133812240e2bf511df4f90a231661f511502868a8b9803</t>
+          <t xml:space="preserve">049525a19d40f882ce415330a1d467ebd26d7e3e641cffe76e19a61ecfeaffaf</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique. Appliquer aussi aux portraits natifs le masque V164 des seules poches de fond admises, en conservant les PNG et le cadrage et en retirant le masque lors de chaque changement de source. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement. </t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-npc-matte-apertures-v164.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
+          <t xml:space="preserve">src/app.js</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">ac0404430bb38a08b454bcc30a4d85a6af1f0afb57a953552739039cdc8180dd</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
+          <t xml:space="preserve">1f0dbf0340728e653b90cb613c8e6676d611e25d0cfedaba15cae2602ac15525</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement. </t>
+          <t xml:space="preserve">Intégrer les propriétaires natifs de circulation, le cycle durable des ascenseurs et la continuité de Lethe dans les vrais hooks du jeu et de ses vues, sans double propriétaire ni action synthétique. Appliquer aussi aux portraits natifs le masque V164 des seules poches de fond admises, en conservant les PNG et le cadrage et en retirant le masque lors de chaque changement de source. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage. Suite V168 : les quatre ouvertures de dialogue désignent leur vrai locuteur et la source de son portrait.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-npc-matte-apertures-v164.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-ui-v163.js</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
+          <t xml:space="preserve">eebe0c5042736c6eeba51b6199946938e6bae7d8483901b78dc8f234c03341e1</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -2233,7 +2233,7 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
+          <t xml:space="preserve">src/campaign-lethe-continuity-v163.js</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
+          <t xml:space="preserve">fea5be5799000bcea712a78685d5cbd54c5ae9ffbe3d55b05692d8809f4aceb7</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -2260,7 +2260,7 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/costume-ui-v119.js</t>
+          <t xml:space="preserve">src/campaign-lethe-story-v163.js</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -2270,24 +2270,24 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a113a45cb2dadc48b88a8835249d8078968eac4642514b7599cdedae4b15e4a</t>
+          <t xml:space="preserve">956cf8bbec54401cce20d8f90ff216c8c6ea951b590cf4d2a2b562f89a1a4d35</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">Étendre la continuité narrative jouable et les retours persistants au-delà des seules histoires QZ18/APC, en conservant moteur natif, compatibilité et paiements stricts. Les insertions C12 exigent leurs vrais contrôles de briefing dans le pilote convoi ; la reprise QZ18 borne seulement les horloges des cinq identités de circuits V163 au temps réel mesuré. Le titre PRÉPARATION débordait du panneau et la disposition portrait héritée réduisait toute l’insertion dans une rangée flex : la CSS dimensionne le titre selon son panneau et donne au flux de lecture la pleine largeur et son vrai défilement vertical, tout en conservant la toolbar et le retour au layout de jeu quand l’insertion disparaît. Le vérificateur natif contrôle conteneurs, textes, vrais viewports et accès aux deux actions par roulette, sans substituer une capture recadrée à la mise en page réelle. L’action PHOTOGRAPHIER, frère absolu du composant, passe également dans le flux après la lecture pendant l’insertion afin de ne plus recouvrir son kicker mobile ; la QA exige son absence de recouvrement et son accès natif par défilement. </t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/franchise-costumes-v119.js</t>
+          <t xml:space="preserve">src/costume-ui-v119.js</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">147afb5919da23a0fda98409ef8914484938786e05f78f1936fe4813e52e32ef</t>
+          <t xml:space="preserve">4a113a45cb2dadc48b88a8835249d8078968eac4642514b7599cdedae4b15e4a</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
@@ -2314,7 +2314,7 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/game-v52-runtime.js</t>
+          <t xml:space="preserve">src/franchise-costumes-v119.js</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -2324,78 +2324,78 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac0049ef9ba4a732b126d2de85984e78e74a9fbef2ca36b428d0fbcf23fa821f</t>
+          <t xml:space="preserve">147afb5919da23a0fda98409ef8914484938786e05f78f1936fe4813e52e32ef</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
+          <t xml:space="preserve">src/game-v52-runtime.js</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7112bc41d7952df2fc4affac5005613d7727041caba8ef5ec5a50e00aec70524</t>
+          <t xml:space="preserve">ac0049ef9ba4a732b126d2de85984e78e74a9fbef2ca36b428d0fbcf23fa821f</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-bulkhead-depth-v134.js</t>
+          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b330fdbf92aa34f8cfb49b58a9229bdedbf4a17ec11663d9ae6e2146a1eec41b</t>
+          <t xml:space="preserve">7112bc41d7952df2fc4affac5005613d7727041caba8ef5ec5a50e00aec70524</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-game.js</t>
+          <t xml:space="preserve">src/hub-batch-command-v168.js</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -2405,24 +2405,24 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e6c4101e04579252bc6045e22cb9305921fbe20c931072732d9a9e045e15b3e</t>
+          <t xml:space="preserve">a22742ea67ac764238a61d317002334e20cce5c83aef538bb20494b8ce974f06</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : protéger les champs de saisie et consommer la touche native d’interaction avant l’ouverture et le focus synchrones du dialogue du refuge, afin que son action clavier par défaut ne rajoute pas un e au nom relu ; conserver les autres contrôles du moteur.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-interaction-input-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
+          <t xml:space="preserve">src/hub-batch-engineering-v168.js</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -2432,51 +2432,51 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">05c6efb9553eb7908a633b1c811651efe6c292c4a036c2f8628fa051c1bae824</t>
+          <t xml:space="preserve">7536e792821110d9f7a24772bb61b4ee662c62d6b4f81596e4671c0dc7eec156</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-life-v136.js</t>
+          <t xml:space="preserve">src/hub-batch-habitat-v168.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ee7433e6b7d663d4c4cee0da5a366617b0141cafad0a63e0928e4924e3b6b7f3</t>
+          <t xml:space="preserve">ae3b1dc39ac8e7818fd3af621cd7d6fa75e7c8ffeacb40514b171405cca8e7ea</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-service-details-v165.js</t>
+          <t xml:space="preserve">src/hub-batch-industrial-v168.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -2486,24 +2486,24 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b6eb5e20ca9c221399135afa5b5fc48d471df74daf9625c194fefe16099037b2</t>
+          <t xml:space="preserve">de153c381e5b32ef05aa420142206323f6102a9b22d3f52d3b75cfb1b56ee1ce</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-v81-runtime.js</t>
+          <t xml:space="preserve">src/hub-bulkhead-depth-v134.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2513,24 +2513,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">26a75cc4fe0e7280146b370c9183cd89a52dabddd865f408289439fe824e4067</t>
+          <t xml:space="preserve">b330fdbf92aa34f8cfb49b58a9229bdedbf4a17ec11663d9ae6e2146a1eec41b</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
+          <t xml:space="preserve">src/hub-game.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2540,24 +2540,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5c9283b4f848a9a5882809f7b4f3c8c84478ed756f89bdc329cd1b875e8e0fe6</t>
+          <t xml:space="preserve">2e6c4101e04579252bc6045e22cb9305921fbe20c931072732d9a9e045e15b3e</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : protéger les champs de saisie et consommer la touche native d’interaction avant l’ouverture et le focus synchrones du dialogue du refuge, afin que son action clavier par défaut ne rajoute pas un e au nom relu ; conserver les autres contrôles du moteur.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-interaction-input-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
+          <t xml:space="preserve">src/hub-lift-transit-v163.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2567,105 +2567,105 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
+          <t xml:space="preserve">05c6efb9553eb7908a633b1c811651efe6c292c4a036c2f8628fa051c1bae824</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
+          <t xml:space="preserve">Replace instantaneous native player deck change with an interruptible approach and durable four-stage trip, preserving native deck/room authority, resources and room projection. Refuse already occupied arrivals and allow a durable same-source cabin return if occupancy blocks a trip before its covered handoff. Detached arrival queries reproduce native annex exclusions and idle spacing before overlaying the actual physical owners, avoiding raw-template false reservations. Keep the native on-screen interact action available during exclusive lift control so touch users can abandon boarding or reopen a source cabin too; query source occupancy only while boarding. Exit via real visible control immediately after trusted cancellation, before observation/PNG I/O consumes the native0.65s return; exact durable return/reload assertions preserved. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/legacy-operations-v131.js</t>
+          <t xml:space="preserve">src/hub-room-backgrounds-v168.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
+          <t xml:space="preserve">4e3821fa5c2dc378c7f8e6e41cfa3126c61a307392df44e18b91c3842e85a21e</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/hub-room-batch-details-v168.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
+          <t xml:space="preserve">e2c9eb8b6e291a0fc685021dc3df17b635e153951c59744e06834a0eb1e7bc51</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/hub-room-life-v136.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">61c15a13031a7d25208a366d1e4f0975b71c317ae23edbf5493778f56f6fa05b</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
+          <t xml:space="preserve">e4d6da6506eec8f9071850079dbf156270895f6fa22395b49dfe8cdf96fb79a2</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
+          <t xml:space="preserve">src/hub-room-parallax-v134.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2675,24 +2675,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
+          <t xml:space="preserve">0b28d10ce68b581b25d2332570155caff802c6249c30c59297b97dcc79d378d3</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
+          <t xml:space="preserve">src/hub-room-service-details-v165.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2702,24 +2702,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
+          <t xml:space="preserve">b6eb5e20ca9c221399135afa5b5fc48d471df74daf9625c194fefe16099037b2</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
+          <t xml:space="preserve">src/hub-v81-runtime.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2729,24 +2729,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
+          <t xml:space="preserve">26a75cc4fe0e7280146b370c9183cd89a52dabddd865f408289439fe824e4067</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/human-patrol-animation-v133.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2756,24 +2756,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
+          <t xml:space="preserve">5c9283b4f848a9a5882809f7b4f3c8c84478ed756f89bdc329cd1b875e8e0fe6</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
+          <t xml:space="preserve">src/human-visual-contract-v133.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2783,105 +2783,105 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
+          <t xml:space="preserve">f009c9e00a60a06cf0cb9d6ecfce22b59d59cfcb8a28d4a9e224d1163abff4c8</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Faire passer les atlas humains par la correction V164 des poches opaques explicitement admises, tout en conservant géométrie, vêtements et garanties RGB du noyau V134. </t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-circulation-v158.js</t>
+          <t xml:space="preserve">src/legacy-operations-v131.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
+          <t xml:space="preserve">70d94552c2614f667fdd5083ee5677249dc733060855329c4551591f048fec60</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
+          <t xml:space="preserve">ab9d4021dde9dcf8609f1a23e43643b0d4f94857836f9df8145641537ce0328d</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
+          <t xml:space="preserve">Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
+          <t xml:space="preserve">scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">058201fe659b0d022f2d29dbde309bdd0ca5efe263c3fa76af54dec65198a010</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
+          <t xml:space="preserve">1e8b4c42e6b5115ff75e86c50dbace7d649c8a4b244629c7788b963a6c690dc5</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Conserver le focus et l’état natif des contrôles lors des scènes originales et des échecs atomiques de stockage, en cohérence avec les nouveaux protocoles C12/Cocon et les retours de campagne. </t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">85a4805f83ddaee04d830a80ca070d3903d7f5933720f859ffd5f7ca489f77c1</t>
+          <t xml:space="preserve">5062de6ccd88582691498bf7c340e9381602937aa1e22f8583efaf308aa60818</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">Correction ciblée de l’affichage hérité du détecteur : proposer une position sous un acteur haut à 320 px lorsque les deux coins HUD le recouvrent, sans modifier les mesures, les contacts ou le comportement du détecteur. Vérification par le profil motion-tracker-v160 déjà obligatoire ; aucun nouveau détecteur ni profil de recette. </t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-leases-v163.js</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
@@ -2891,34 +2891,34 @@
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
+          <t xml:space="preserve">e133273662735daeff048498358ea3f56744acb9db2af540f196cd5f7a1bb123</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-life-v136.js</t>
+          <t xml:space="preserve">src/npc-annex-service-routes-v163.js</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
+          <t xml:space="preserve">25d7efed89dc1134a79cabe8fad259c029c2db8db58f43d1a2fa4be487a0f92f</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
@@ -2935,7 +2935,7 @@
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
+          <t xml:space="preserve">src/npc-annex-workpost-routes-v165.js</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
+          <t xml:space="preserve">b9bf2fca2a46fa79e11fc9f467c1672c11d33e8c4922ee8afbfcc6a48fb5fafe</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
@@ -2962,7 +2962,7 @@
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
+          <t xml:space="preserve">src/npc-cal-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
@@ -2972,24 +2972,24 @@
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
+          <t xml:space="preserve">2ac8b1c472c20689772ddfe35199e49bd2125b6d3e90237f8c6da2d4ccc2813d</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
+          <t xml:space="preserve">src/npc-cal-logistics-route-v165.js</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
@@ -2999,78 +2999,78 @@
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
+          <t xml:space="preserve">e8206918faeede321fac0b43275da1a62a80e9591c7ff97b86ec8cf9ed7f5acc</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="41" ht="48" customHeight="1">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
+          <t xml:space="preserve">src/npc-circulation-v158.js</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">8ba022817afb11bec4bb9af5056982ccadd63f4707f0859cc40bd94c431252fa</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
+          <t xml:space="preserve">9a113b6f54dc273da215fdb3c03f12b8e9471a9475b4f9eb275b6b56b6ac4a99</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
+          <t xml:space="preserve">src/npc-dialogue-portraits-v168.js</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
+          <t xml:space="preserve">04a7f8db4f4bb7bd10b2da6d90b8a0e20f647c3c9d0b6123fee77fd65d1b56c7</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
+          <t xml:space="preserve">src/npc-interdeck-passage-v165.js</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
@@ -3080,24 +3080,24 @@
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
+          <t xml:space="preserve">d2db8cee7f823db24a79f6125dbe06cf872b05344995bcb2d7a14e42e9bcdd9f</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
+          <t xml:space="preserve">src/npc-interdeck-routes-v165.js</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
+          <t xml:space="preserve">85a4805f83ddaee04d830a80ca070d3903d7f5933720f859ffd5f7ca489f77c1</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
@@ -3124,88 +3124,88 @@
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
+          <t xml:space="preserve">src/npc-jun-climb-rig-v165.js</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
+          <t xml:space="preserve">75d5d7a0a8cbf82a3fdf9569713bc921badd40834ee9c43f8f479802174330a0</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
+          <t xml:space="preserve">src/npc-life-v136.js</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">6179892f6f37f1220c85de66bc5ac0bd94fce15ea8d643d6dd53b2280735ebb3</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
+          <t xml:space="preserve">ccd320fd541abf156e59cac8e2af45322b908204e5141849252de487102c66d9</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. </t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs</t>
         </is>
       </c>
     </row>
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
+          <t xml:space="preserve">src/npc-lift-transit-v165.js</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
+          <t xml:space="preserve">2b492180395b6d78a73414a345a89c109f796daf3e18644b7b8419db223cd55b</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
+          <t xml:space="preserve">src/npc-matte-aperture-data-v164.js</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
@@ -3215,24 +3215,24 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
+          <t xml:space="preserve">d0216d395ee7f861d9ecb89db955833f34cd97bdd9aa6ad5133702819b6195da</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">Épingler les sources et runs exacts de poches de fond explicitement admises dans seize cellules de quatre PNJ, sans redessiner les PNG ni certifier leurs autres poses. </t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-v126.js</t>
+          <t xml:space="preserve">src/npc-matte-apertures-v164.js</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
@@ -3242,24 +3242,24 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
+          <t xml:space="preserve">588c9350e2a0936ef11f7287521f98325650fee7f71401543641dad5a234b9fb</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">Corriger les seuls pixels opaques de fond admis avec garde des octets ciblés, cache borné et gestion des changements de portrait sans clé globale des blancs. </t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-matte-apertures-v164.mjs</t>
         </is>
       </c>
     </row>
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
+          <t xml:space="preserve">src/npc-mission-runtime-v55.js</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
@@ -3269,51 +3269,51 @@
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
+          <t xml:space="preserve">d1922839a7e23f9912ae2e38d5e2ae442cf6da67718ae0e97d28d5fc4f5b6390</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
+          <t xml:space="preserve">src/npc-service-routes-v161.js</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3bfd466c91a0861b1f99c806769a69a144942627c25fe2f1d47dcbd40711bf56</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
+          <t xml:space="preserve">d3a3c9e274dbf5a92d930c39583bb2a056ead0c1c5d0f9162ee6e632ccf70750</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
+          <t xml:space="preserve">src/npc-service-traffic-v163.js</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
@@ -3323,132 +3323,132 @@
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
+          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/npc-station-relays-v166.js</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
+          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-climb-rig-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
         </is>
       </c>
     </row>
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
+          <t xml:space="preserve">7f056e474636f829e5309b1c52e68e04d3e2844b275fb001b574d6af90fb8b6f</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-appearance-preview-v126.js</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2fef117a684b16b6c426ed93f932ce91e660648682f50600c799f5cd6126c8f9</t>
+          <t xml:space="preserve">92dd0643f85d4eee5a4daaab6e425b5e4ca68097a6f31e2e792f3e6674da96e0</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">3ab7e4155ca7ac97dd447c25df168374c815ea1eee07370f9674d3a8ccd12bf0</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
+          <t xml:space="preserve">cce67f9128241fcf6e8f6932a57ec73b080c7e875acf024e15259450dbd9188b</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active.</t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/player-appearance-ui-v126.js</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
@@ -3458,51 +3458,51 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">413261d7c85d408b4e08ccd46bc0d2e6ea4fca7ac64bed5bf73ef6d1c6bf859a</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/player-appearance-v126.js</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
+          <t xml:space="preserve">69c62a380a15d2d3b34e950620cd514fa780b531d016071029a17215c5ee59e1</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
+          <t xml:space="preserve">src/player-costume-atlases-v165.js</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
@@ -3512,24 +3512,24 @@
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
+          <t xml:space="preserve">4026d6e6b6047a7d868d2b03cea56da3e2dd5de7f099ac730a0166a3b844a8e6</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions.</t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/player-costume-outfits-v165.js</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
@@ -3539,24 +3539,24 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/player-costume-parts-v165.js</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
@@ -3566,105 +3566,105 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">9e0a9c7a60e95a4a862b2345bae0f2e29f9546f30e9435e1b7538f5a3695a7de</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">719b3fc6a0e9efa876d640f292794fc1766ceb646b7d74effb6914e4419f2cb0</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">2fef117a684b16b6c426ed93f932ce91e660648682f50600c799f5cd6126c8f9</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+          <t xml:space="preserve">src/refuge-art-v87.js</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
@@ -3674,24 +3674,24 @@
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
@@ -3701,150 +3701,393 @@
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage. Suite V168 : les quatre ouvertures de dialogue désignent leur vrai locuteur et la source de son portrait.</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="71" ht="48" customHeight="1">
       <c r="A71" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="48" customHeight="1">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="48" customHeight="1">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="48" customHeight="1">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="48" customHeight="1">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V162</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="48" customHeight="1">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="48" customHeight="1">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="48" customHeight="1">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+        </is>
+      </c>
+      <c r="D78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="48" customHeight="1">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B71" s="0" t="inlineStr">
+      <c r="B80" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
-      <c r="C71" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">f51ae4141ecbf889dfd79261f0442d46f8b5b837e0038f8e8291ad157c604e6b</t>
-        </is>
-      </c>
-      <c r="D71" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165. Suite V167 : nouveau cache des mouvements humains et plaques de portes.</t>
-        </is>
-      </c>
-      <c r="E71" s="0" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">732d8eca7c6a8e4443f5a4d26b6a4cd677f2ad5b3fc1c4e766b452606ce153e9</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165. Suite V167 : nouveau cache des mouvements humains et plaques de portes. Suite V168 : précacher les sept modules de portraits et de décor dans un namespace distinct.</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
@@ -25639,7 +25882,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Révision des appuis et attaches du bassin, des jambes et du torse ; cadence liée à la distance, continuité marche/arrêt et présentation des humains alliés. Suite V167 : bras mains libres synchronisés aux pas ; continuité des alliés à travers les actions et rejet des faux pas sans temps écoulé.</t>
+          <t xml:space="preserve">Révision des appuis et attaches du bassin, des jambes et du torse ; cadence liée à la distance, continuité marche/arrêt et présentation des humains alliés. Suite V167 : bras mains libres synchronisés aux pas ; continuité des alliés à travers les actions et rejet des faux pas sans temps écoulé. Suite V168 : seize portraits individuels tête/épaules dans les cadres de dialogue, sans nouveau PNG.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -25649,12 +25892,12 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/human-patrol-animation-v133.js ; src/sprite-animation-runtime.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/human-patrol-animation-v133.js ; src/sprite-animation-runtime.js ; src/npc-dialogue-portraits-v168.js</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/qa-player-allies-contacts-v165.py</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs ; scripts/qa-player-allies-contacts-v165.py</t>
         </is>
       </c>
       <c r="H10" s="0">
@@ -25682,7 +25925,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 assemblages de service pour 35 profils de pièces ; quatre vues volontairement dégagées. Plaque du vrai nom sur le cadre du refuge ; retrait des gros libellés de développement. Suite V167 : plaques physiques de destination fixées aux douze linteaux, dans les deux projections.</t>
+          <t xml:space="preserve">31 assemblages de service pour 35 profils de pièces ; quatre vues volontairement dégagées. Plaque du vrai nom sur le cadre du refuge ; retrait des gros libellés de développement. Suite V167 : plaques physiques de destination fixées aux douze linteaux, dans les deux projections. Suite V168 : lot001 de cent installations, quatre secteurs de vingt-cinq, trente-six types, et trente-cinq profils de fond ; aucune collision nouvelle.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -25692,12 +25935,12 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hub-room-service-details-v165.js ; src/hub-room-life-v136.js ; src/refuge-art-v87.js ; src/hub-bulkhead-depth-v134.js</t>
+          <t xml:space="preserve">src/hub-room-service-details-v165.js ; src/hub-room-life-v136.js ; src/refuge-art-v87.js ; src/hub-bulkhead-depth-v134.js ; src/hub-room-backgrounds-v168.js ; src/hub-room-batch-details-v168.js ; src/hub-batch-command-v168.js ; src/hub-batch-habitat-v168.js ; src/hub-batch-industrial-v168.js ; src/hub-batch-engineering-v168.js</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/qa-hub-service-details-v165.py</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs ; scripts/qa-hub-service-details-v165.py ; scripts/qa-tantalus-batch100-v168.py</t>
         </is>
       </c>
       <c r="H11" s="0">

</xml_diff>

<commit_message>
fix: preserve refuge glass and account for rendered batch atlas props
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -2594,7 +2594,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4e3821fa5c2dc378c7f8e6e41cfa3126c61a307392df44e18b91c3842e85a21e</t>
+          <t xml:space="preserve">c9ce994af2a7d053790f445c4023492764ffd083836fbad362f34ef32b4862d4</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e2c9eb8b6e291a0fc685021dc3df17b635e153951c59744e06834a0eb1e7bc51</t>
+          <t xml:space="preserve">f940cf464baa31c21440f30e17b3d2a2eb1389008e14c5ce6b3aa877eae28068</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix: place all100 ship details around live traversal reservations
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a22742ea67ac764238a61d317002334e20cce5c83aef538bb20494b8ce974f06</t>
+          <t xml:space="preserve">82b773e62e03ba72a99ed161044b43c36f56d3e2756cd795aade1bc2a58dd255</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7536e792821110d9f7a24772bb61b4ee662c62d6b4f81596e4671c0dc7eec156</t>
+          <t xml:space="preserve">b225caf172d8502f5e82c0b13b0b61d5eae8a05d46a77119e34b9de5e23457b9</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ae3b1dc39ac8e7818fd3af621cd7d6fa75e7c8ffeacb40514b171405cca8e7ea</t>
+          <t xml:space="preserve">e245850c5c22ec8be2615d645fdfbc7f975b0e54445b2ff90f04d4010c6c50dd</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">de153c381e5b32ef05aa420142206323f6102a9b22d3f52d3b75cfb1b56ee1ce</t>
+          <t xml:space="preserve">2e8b216d47285646aa46920f584577e2e249e85e8c22734bcb16a65585bb419c</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix: clear visible pipework and identify wall-mounted equipment
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">82b773e62e03ba72a99ed161044b43c36f56d3e2756cd795aade1bc2a58dd255</t>
+          <t xml:space="preserve">417014faf4c286174285c16bcb6a4f16f26720ee315dd19e03085bfc73485fd1</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e245850c5c22ec8be2615d645fdfbc7f975b0e54445b2ff90f04d4010c6c50dd</t>
+          <t xml:space="preserve">8553034ff4821accbb8651b868ead51d434458ecda5f9a16a2b8936f0c7dddaa</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f940cf464baa31c21440f30e17b3d2a2eb1389008e14c5ce6b3aa877eae28068</t>
+          <t xml:space="preserve">e5093cef235c0e7531bb20d9f067b99e38e4a32f60f07e6de21761f5022e0a9b</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix: débloquer les files PNJ et fiabiliser les parcours natifs
Étendre les réservations de dégagement aux pairs admissibles qui occupent les baies proposées, en conservant les gardes atomiques et la marche native.

Corriger les observations QA de dessin d’arme, d’amarrage et de sortie d’échelle. Couvrir les régressions avant/après, la reprise des trajets et les refus natifs.

Actualiser les empreintes courantes et les deux cellules de succession du classeur avec son générateur déterministe ; conserver les historiques et les limites de validation navigateur.
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -3323,12 +3323,12 @@
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">08d91c32f20217f1f3eb9f193787f17096745e304e8c48287a633c789ea95147</t>
+          <t xml:space="preserve">9279832e7d9f8a13191c57f84c564c16655c3ff79defeead08246154f73e5cdb</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées. Maintenance gamedev du 29 octobre 2026 : inclure les pairs admissibles qui occupent une baie de dégagement proposée, jusqu’à stabilisation de la chaîne ; préserver ordre physique, identités, garde atomique, préemptions autorisées et reprise.</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix: coordonner les propriétaires PNJ et fiabiliser sept parcours natifs
Permettre à Tamsin de dégager physiquement le trajet de Maksim sous son propriétaire V166, avec le plan collectif, les priorités, les collisions et la reprise existants.

Corriger les parcours QA d’Idris, Echo, Asha, Inez, Amanda et Trials pour attendre la bonne cible, la vraie dépendance physique et le même événement de capture. Préserver les gardes et documenter les actions natives et les doubles utilisés.

Valider 158 tests ciblés, dont 23 nouveaux, et les reproductions natives avant/après. Régénérer le classeur et les empreintes cumulatives en conservant les historiques et les reçus antérieurs. Documenter séparément le blocage navigateur de Jun encore non résolu.
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -3323,12 +3323,12 @@
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9279832e7d9f8a13191c57f84c564c16655c3ff79defeead08246154f73e5cdb</t>
+          <t xml:space="preserve">50b90764828ab341cabb0d5795addd06092beed00957e6abc2a8310675e8de5d</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées. Maintenance gamedev du 29 octobre 2026 : inclure les pairs admissibles qui occupent une baie de dégagement proposée, jusqu’à stabilisation de la chaîne ; préserver ordre physique, identités, garde atomique, préemptions autorisées et reprise.</t>
+          <t xml:space="preserve">V162 contained only four physically observed annex circuits; native timetable bodies appeared in other annexes without real observed travel. V163 adds five real bounded circuits and resolves actual native watch lane conflicts. A naive virtual createNpcs peer probe re-admitted lifecycle owners; pure RoutineHub sampling and exact actual-owner replacement preserve historical161/162 invariants. Three additional same-deck annex watches are now physical leases of their existing historical owners, avoiding duplicate crew identities and avoiding invented NPC lift/climb travel. The real05h30 exit →09h30 command-screen routine rebuild →restart of the saved hub also requires retaining the ECHO V158 supported source bookmark until its first native-frame lease admission, before any new annex post can replace that origin. The exact d180 Jun native-annex receipt exposed a physical collision-owner omission: generic route tick suppression also hid Jun from Pablo collision peers, allowing their same-floor bodies to overlap. V163 now gives ordinary annex life the unfiltered exact-singleton physical cohort while retaining its existing filtered movement iteration, and skips the ordinary tick for leased owners so only the lease advances occupation. The QA approach respects the real station-priority72px boundary and physical crew spacing, waits for measured native patrol progress when every approach is occupied, and still requires the exact requested speaker. V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées. Maintenance gamedev du 29 octobre 2026 : inclure les pairs admissibles qui occupent une baie de dégagement proposée, jusqu’à stabilisation de la chaîne ; préserver ordre physique, identités, garde atomique, préemptions autorisées et reprise. Quatrième application gamedev du 29 octobre 2026 : réserver dans le plan collectif une baie physique pour Tamsin avant son premier service lorsque le véritable trajet Maksim-cockpit traverse le pont 0 ; conserver son propriétaire V166, son corps unique, son origine observée et les phases durables de dégagement, attente et retour, avec refus atomiques, collisions, priorités et cloisons natives.</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -3350,12 +3350,12 @@
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e0fc98ade1450bd4fa82e1de513172fb8573bc4932d2c0722e77e9311437e8f1</t>
+          <t xml:space="preserve">371f5de036111531b79adffea4e6d5ffaf0c1f86f5773b18fed88b129ccaf156</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées.</t>
+          <t xml:space="preserve">V165 : étendre les propriétaires PNJ existants avec deux boucles locales, le trajet vertical logistique de Cal et les contrôleurs de service inter-ponts ; conserver corps unique, appuis, réservation des cabines, fermeture des portes, interruptions et reprise durable sans créditer de trajet non observé. Suite V167 : conserver le corps réellement observé pendant un changement stratégique sans temps physique et réhydrater les propriétaires de la sauvegarde avant tout ancien cohort du moteur réutilisé. Suite V166 : relier physiquement les postes capteurs de Rook et briefing de Tamsin à leurs services locaux, partager les cabines, rendre le même corps et son origine après service ; préserver sauvegardes, courtoisies réelles et portes verrouillées occupées. Quatrième application gamedev du 29 octobre 2026 : réserver dans le plan collectif une baie physique pour Tamsin avant son premier service lorsque le véritable trajet Maksim-cockpit traverse le pont 0 ; conserver son propriétaire V166, son corps unique, son origine observée et les phases durables de dégagement, attente et retour, avec refus atomiques, collisions, priorités et cloisons natives.</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">

</xml_diff>

<commit_message>
feat: intégrer les tenues Vasquez et Rain et fiabiliser le parcours Jun
Ajouter quatre atlas documentés, leurs pièces et variantes directionnelles, puis corriger le pilote natif Jun pour le conduit et le dialogue. Conserver les limites de fidélité et les preuves ciblées dans le guide et le suivi.
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V163.xlsx
@@ -122,8 +122,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E80" totalsRowShown="0">
-  <autoFilter ref="A5:E80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV163Table11" displayName="AuditV163Table11" ref="A5:E81" totalsRowShown="0">
+  <autoFilter ref="A5:E81"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V162"/>
@@ -3539,12 +3539,12 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed0e7d794aecfa733a9e271611cc7d7928deea3b1e72fa4d7a2ed170a95d01bd</t>
+          <t xml:space="preserve">9a28b82d1dabd95c926052d85d7aaccbc25a32abd96e8590d8a7b6d365da7f42</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : ajouter les tenues modulaires Vasquez BDU et Rain au catalogue, aux six emplacements et aux transactions existantes ; réutiliser le bandeau V129 sous son identifiant historique sans dupliquer son entrée. Conserver les armes choisies, les sauvegardes, les dix autres ensembles modulaires et le statut d’adaptation non certifiée.</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">94f3cba4aa29950b749fad9e0a109dae8573d09e34f44d91db80c1814ddc8195</t>
+          <t xml:space="preserve">7913947158b5ad5431f09f151009069060a49fdbfa94d71598d11caad7eb74b3</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : raccorder huit créations de tenues en pièces modulaires à la personnalisation de l’opérateur et lier Hicks/Hudson à leurs vrais presets V129 existants ; distinguer les dix-sept PNG de pièces portables des quinze atlas de référence et conserver le skin Nostromo historique, équipement, identité et compatibilité des anciens profils.</t>
+          <t xml:space="preserve">V165 : intégrer quatre PNG originaux transparents pour Vasquez BDU et Rain, six poses de torse par tenue et deux orientations des chaussures de Rain. Mesurer les découpes, ouvertures et appuis, puis recaler les épaules sur des rendus des vrais pixels. Préserver exactement les huit kits antérieurs et leurs dix-sept fichiers ; les nouveaux vêtements restent adaptés à Echo9, sans certification 1:1.</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -3664,34 +3664,34 @@
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/refuge-art-v87.js</t>
+          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
+          <t xml:space="preserve">62a3b7466b5d851c95d31ef00da7e79d8b65f43c0331e9a9d7acbe960a8f3103</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
+          <t xml:space="preserve">V165 : sélectionner une définition gauche complète lorsqu’elle existe et respecter l’orientation source des chaussures de Rain pour conserver le sens du marquage. Garder les calculs antérieurs pour les pièces sans variante, refuser une variante présente mais incomplète et conserver les appuis, l’IK, la physique et les transitions de locomotion.</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-transit-rig-v128.mjs ; scripts/verify-player-locomotion-rig-v129.mjs</t>
         </is>
       </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/reload-presentation-v163.js</t>
+          <t xml:space="preserve">src/refuge-art-v87.js</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
@@ -3701,78 +3701,78 @@
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
+          <t xml:space="preserve">958f9c403d5dab828df67781425afe120769b45666f2e2a51732339b5831f053</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : poser trente et un assemblages techniques sur les seules baies libres des murs arrière des trente-cinq pièces, avant le mobilier natif, avec réservations et projection de la pièce ; intégrer le nom choisi sur le cadre du refuge sans légende de développement ni modification des collisions ou portes. Suite V167 : fixer la signalétique de destination au linteau des douze cloisons selon leur projection, sans changement de collision ou de trajet ; transmettre la touche de dialogue à Tamsin dans le stand hors qualification active. Suite V168 : cent installations murales choisies par usage, trente-cinq fonds architecturaux et suppression des retours obliques dans les sections frontales ; conserver les réservations, dimensions, pixels existants, géométrie et projection de chaque pièce.</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-hub-service-details-v165.mjs ; scripts/verify-ship-placement-v167.mjs ; scripts/verify-range-crew-interaction-v167.mjs ; scripts/verify-tantalus-batch100-v168.mjs ; scripts/verify-hub-backgrounds-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/reload-presentation-v163.js</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
+          <t xml:space="preserve">1d7611f540bd44b74f4ac9457026a59824fd30b06cf24d2ffb4b6cbc37963bce</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage. Suite V168 : les quatre ouvertures de dialogue désignent leur vrai locuteur et la source de son portrait.</t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
+          <t xml:space="preserve">src/save.js</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non épinglé en V162</t>
+          <t xml:space="preserve">98a20e4a0f52a7c33d5d3e53757ad4aba30cad350bacbe2fbac4aa8a6dc3403a</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
+          <t xml:space="preserve">afd5b289887c3a6be5d704ad9b501d9cd7bfeae4514fdfb4eaf21095e6d42304</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
+          <t xml:space="preserve">Déclarer et normaliser les états durables de continuité de campagne, circuits d’annexes, courtoisie physique et trajet joueur ascenseur tout en conservant la reprise des sauvegardes historiques. V165 : intégrer et sérialiser les propriétaires de service PNJ, les pièces de costumes et les présentations effectivement atteintes par la production ; préserver les transactions, les interruptions, la normalisation des sauvegardes et l’unicité des corps, sans changer le schéma public ni attribuer des preuves futures. Suite V166 : intégrer et normaliser les propriétaires des deux trajets de poste sans dupliquer les corps ni inventer un voyage. Suite V168 : les quatre ouvertures de dialogue désignent leur vrai locuteur et la source de son portrait.</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-lethe-v163.mjs ; scripts/verify-campaign-story-v160.mjs ; scripts/verify-npc-annex-service-routes-v163.mjs ; scripts/verify-npc-service-routes-v161.mjs ; scripts/verify-npc-medical-route-v162.mjs ; scripts/verify-npc-annex-leases-v163.mjs ; scripts/verify-npc-life-v136.mjs ; scripts/verify-npc-circulation-v158.mjs ; scripts/verify-npc-annex-circulation-v159.mjs ; scripts/verify-hub-lift-transit-v163.mjs ; scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs ; scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs ; scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-npc-annex-workpost-routes-v165.mjs ; scripts/verify-npc-cal-logistics-route-v165.mjs ; scripts/verify-npc-interdeck-routes-v165.mjs ; scripts/verify-npc-interdeck-passage-v165.mjs ; scripts/verify-npc-jun-climb-rig-v165.mjs ; scripts/verify-npc-station-relays-v166.mjs ; scripts/verify-npc-relay-locked-bulkheads-v166.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
+          <t xml:space="preserve">src/sprite-animation-runtime.js</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
@@ -3782,24 +3782,24 @@
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
+          <t xml:space="preserve">33a86ab323c4694b670334a12cc89273c5953bcde8bccb21a0115b8bebe19d01</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
+          <t xml:space="preserve">V165 : resserrer et raccorder les appuis, les longueurs de membres et les attaches du joueur et des alliés, avec marche entraînée par le déplacement réel, transitions et secours de chargement ; les corps physiques et les armes demeurent les propriétaires natifs. Suite V167 : synchroniser les bras mains libres avec les pas observés ; rejeter les déplacements à horloge figée et conserver la phase de marche des alliés pendant leurs actions au sol, sans modifier les événements de ces actions. Suite V168 : cadrer les seize vrais locuteurs sur leur tête et leurs épaules, avec transparence conservée, initiales accessibles et protection contre les chargements tardifs ; ne jamais présenter un sprite entier comme avatar.</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-allies-contacts-v165.mjs ; scripts/verify-player-locomotion-rig-v129.mjs ; scripts/verify-player-appearance-v126.mjs ; scripts/verify-player-arm-phase-v167.mjs ; scripts/verify-allied-patrol-phase-v167.mjs ; scripts/verify-dialogue-portraits-v168.mjs</t>
         </is>
       </c>
     </row>
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
+          <t xml:space="preserve">src/weapon-effects-runtime-v124.js</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
@@ -3809,24 +3809,24 @@
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
+          <t xml:space="preserve">7a47a03249fc2e45390608bf95f8496846da83cca0714d7f4b9b8657b28d1bfb</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
+          <t xml:space="preserve">Défaut reproduit avec vrai V77 : à54% le secondR PERFECT change elapsed/completeAt de.54 à.7714, sauteinsert→seat et déplace instantanément la main M41A de17.162514px. Le helper corrige tous les feeds sans modifier la transaction. </t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-reload-presentation-v163.mjs ; scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-runtime-v124.mjs ; scripts/verify-weapon-effects-v124.mjs</t>
         </is>
       </c>
     </row>
     <row r="71" ht="48" customHeight="1">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-data-v163.js</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
+          <t xml:space="preserve">f73824fd19bb4b26169583e038b9a272051d25cbdb6556c45f560f968866a285</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
@@ -3853,7 +3853,7 @@
     <row r="72" ht="48" customHeight="1">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-capture-v163.js</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
+          <t xml:space="preserve">2c7fb5a5111e6d2ddf5b89baa5232dc613767708ed523fc531a2ea72657cf775</t>
         </is>
       </c>
       <c r="D72" s="0" t="inlineStr">
@@ -3880,7 +3880,7 @@
     <row r="73" ht="48" customHeight="1">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
+          <t xml:space="preserve">src/xeno-trials-engine-v96.js</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
+          <t xml:space="preserve">48e4e6cc8091e2f266f0b6831eb5d08f523a9acc27ba1f23cea3f227aaf0a007</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
@@ -3907,7 +3907,7 @@
     <row r="74" ht="48" customHeight="1">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
+          <t xml:space="preserve">src/xeno-trials-grapple-v153.js</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
@@ -3917,24 +3917,24 @@
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
+          <t xml:space="preserve">a0d85cfeb6cac1b3b97f0334ca7656c324f43a9077cac04b22600fdf6cc6529a</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. </t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="75" ht="48" customHeight="1">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v163.js</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
@@ -3944,150 +3944,177 @@
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
+          <t xml:space="preserve">4f7dfdd9b88c8effd9192899a6af35806b30f96a3a17c6016a09527e6a09f401</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="76" ht="48" customHeight="1">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-data-v165.js</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
+          <t xml:space="preserve">Non épinglé en V162</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
+          <t xml:space="preserve">396896622c85ff1198c4f61fb0e3a5f5eb131f1d74f315f6cb8aca24d64461d5</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
+          <t xml:space="preserve">V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v165.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
         </is>
       </c>
     </row>
     <row r="77" ht="48" customHeight="1">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-rig-v154.js</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
+          <t xml:space="preserve">8fe2289b2db7860646dbc12d818cf007f3e2b716cfa738b230645eff392dc79c</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
+          <t xml:space="preserve">c380d8b4613ef37cb978880050c37a183b4113bfa7e833817810fc95ef1a93a5</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. V165 : admettre cent soixante-dix rigs de présentation bornée, chacun attaché aux pixels et à l’empreinte de sa propre image native ; préserver les dix-neuf rigs antérieurs et distinguer ces poses des marches complètes, captures et mouvements canoniques non produits.</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-native-rig-catalog-v165.mjs</t>
         </is>
       </c>
     </row>
     <row r="78" ht="48" customHeight="1">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
+          <t xml:space="preserve">src/xeno-trials-runtime-v96.js</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
+          <t xml:space="preserve">4dcf2018e86b072fc9412040b78c872b4b4c8d952a1cccaec0fd7b0e46e71e72</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
+          <t xml:space="preserve">ef87fa84ba5f085cd0fc973b40dfeb11cf832f88b5168e259c2bc406303a2867</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. Les preuves héritées couvrent la migration Broodstorm en tests de proximité et la sortie spatiale sur hôte de rendu ; ces deux priorités requièrent une recette liée au candidat courant avec vrai parcours production/menu/Save. La navigation Retour corrige le clic et le clavier interceptés par la pause de focus, tout en conservant les autres pauses. La revue des vrais pixels Broodstorm d180 a aussi révélé un rectangle opaque de station superposé à Cheyenne et un ancien objectif affiché sous le HUD : le rendu de vol retire ce rectangle, conserve navette et interaction E, masque le doublon et remplace les détails d’implémentation par la consigne CHARGES LIMITÉES, sans changer les limites déclarées dans le dossier/API. </t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs ; scripts/verify-legacy-operations-v131.mjs ; scripts/verify-xeno-trials-presentations-v156.mjs ; scripts/verify-trials-navigation-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="79" ht="48" customHeight="1">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+          <t xml:space="preserve">src/xeno-trials-sequences-v155.js</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+          <t xml:space="preserve">aace792160253b9df4d63e68da39cc20981565b7331607785c27f80ad34440af</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+          <t xml:space="preserve">ed140f0788d4d13b91ddd0aaa8a955c7ca50507185f9eee3debd537385ad2321</t>
         </is>
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+          <t xml:space="preserve">The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+          <t xml:space="preserve">scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
         </is>
       </c>
     </row>
     <row r="80" ht="48" customHeight="1">
       <c r="A80" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/xeno-trials-ui-v96.js</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2c60081f22f1a4853e449c23893c88334a3537aa2be3c81e16c609839ee0212e</t>
+        </is>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afcbe460f875f5f03285a4b2b509bbdebdbba081dd7d18447a33f97a0231568a</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les portraitsdebout natifs ne contenaientaucun corpscouché recevable ; troisnouveauxatlas ImageGen originaux ont été créés à partir desréférenceslocales inspectées, conservésbyteidentiques, sanspivotementrigide ni retouchepixels. Aucunrelevéartistiquecanonique externe nepeutêtreclôturé. Une recette native de capture V163 a ensuite reproduit une résistance CPU déjà engagée (33 ticks) annulée après pause : le masque de réarmement du clavier était appliqué à tort au CPU, qui renouvelait sa garde sans relâche jusqu’au timeout. Le moteur distingue désormais le dernier flux adverse CPU/direct, conserve cette propriété dans les snapshots, traite explicitement le legacy CPU et préserve toutes les contraintes de relâchement des entrées humaines. Le HUD demandait au joueur de maintenir la garde même lorsque le captif était le CPU. Le libellé suit désormais le propriétaire réel du captif, dans la vue accessible comme dans le Canvas, sans changer les prises ni leur évasion. Aligner aussi l’ombre au sol sur la racine et la largeur de la plaque réellement affichée, sans déplacer le corps autoritaire du moteur. The185 non-pilot identities already have static project sprites; admissible anatomy-specific technical rig production can progress without misclassifying those sprites as absent or promoting generic rigs/canonical motion. The native runtimeV96 intro also displayed an undefined family for the existing hybrid identity and placed its fixed card over tall source silhouettes. The targeted corrections add the HYBRIDE label and position the card below the support plane;47 catalogue checks pass, including actual recorded controller intro rendering for all189 identities in both slots (378 intro renders), defined six-family labels, card/text screen bounds and non-overlap with both measured native alpha envelopes. These Node fixtures are distinct from browser raster/final exact-head recipe evidence. </t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-xeno-trials-capture-v163.mjs ; scripts/verify-xeno-trials-rig-v154.mjs ; scripts/verify-xeno-trials-restraint-pose-v156.mjs ; scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-native-rig-catalog-v163.mjs ; scripts/verify-xeno-trials-grapple-v153.mjs ; scripts/verify-xeno-trials-controls-v150.mjs ; scripts/verify-capture-admission-v163.mjs ; scripts/verify-native-rig-terminal-v163.mjs ; scripts/verify-native-rig-weapon-rigidity-v163.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="48" customHeight="1">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B80" s="0" t="inlineStr">
+      <c r="B81" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">0b506c1e7e57e36e50348d3a89400cc5976a65202b8830ef2163f9cde0c2e657</t>
         </is>
       </c>
-      <c r="C80" s="0" t="inlineStr">
+      <c r="C81" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">732d8eca7c6a8e4443f5a4d26b6a4cd677f2ad5b3fc1c4e766b452606ce153e9</t>
         </is>
       </c>
-      <c r="D80" s="0" t="inlineStr">
+      <c r="D81" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Épingler explicitement les modules, styles et trois nouveaux PNG de capture admis pour leur disponibilité hors ligne, sans élargir les règles de publication des preuves privées. Ajouter les deux modules de correction des poches PNJ V164 au shell hors ligne vérifié par le contrôle réel de distribution. Séparer aussi le namespace du worker source V164 du cache actif V163 afin de conserver celui-ci si le nouveau précache échoue. V165 : admettre dans le cache de production les nouveaux modules effectivement intégrés avec un namespace distinct, sans réadmettre les sources privées, les prévisualisations hors périmètre ni les fichiers différés Forge. Suite V166 : séparer le cache des nouveaux trajets de poste du cache V165. Suite V167 : nouveau cache des mouvements humains et plaques de portes. Suite V168 : précacher les sept modules de portraits et de décor dans un namespace distinct.</t>
         </is>
       </c>
-      <c r="E80" s="0" t="inlineStr">
+      <c r="E81" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-public-release-v86.mjs ; scripts/verify-release-artifact-v143.mjs ; scripts/verify-audit-v143.mjs</t>
         </is>
@@ -25710,22 +25737,22 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huit créations de tenues modulaires, dix-sept PNG de pièces portables ; deux liaisons aux vrais presets V129 Hicks/Hudson, soit dix références équipables. Les trois dernières créations adaptent des kits Fireteam documentés distincts. Quinze atlas de référence, 240 cellules, séparés du rendu jouable.</t>
+          <t xml:space="preserve">Dix créations de tenues modulaires, vingt et un PNG de pièces portables ; deux liaisons aux vrais presets V129 Hicks/Hudson, soit douze références équipables dans ce chantier. Vasquez BDU et Rain ajoutent quatre PNG avec torses gauche/droite distincts et chaussures directionnelles pour Rain. Quinze atlas de référence, 240 cellules, restent séparés du rendu jouable.</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20 autres références franchise restent ouvertes. Les deux liaisons réutilisent des vêtements V129 et ne sont pas de nouveaux arts. Nostromo V119 conserve ses cinq PNG ; aucun fallback précomposé à M41A pour les nouveaux kits. Aucune approbation artistique 1:1.</t>
+          <t xml:space="preserve">18 autres références franchise restent ouvertes. Le catalogue complet compte 31 entrées et 13 tenues équipables en incluant le Nostromo V119 historique, hors des 30 références de ce chantier. Les deux liaisons V129 réutilisent des vêtements existants ; les cinq PNG Nostromo restent inchangés. Les nouveaux kits habillent Echo9 et utilisent son arme réellement équipée. Aucune approbation artistique 1:1.</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-costume-atlases-v165.js ; src/player-costume-outfits-v165.js ; src/player-costume-parts-v165.js</t>
+          <t xml:space="preserve">src/player-costume-atlases-v165.js ; src/player-costume-outfits-v165.js ; src/player-costume-parts-v165.js ; src/player-transit-rig-v128.js</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs ; scripts/qa-costume-atlases-v165.py</t>
+          <t xml:space="preserve">scripts/verify-costume-atlases-v165.mjs ; scripts/verify-player-transit-rig-v128.mjs ; scripts/qa-costume-atlases-v165.py</t>
         </is>
       </c>
       <c r="H6" s="0">

</xml_diff>